<commit_message>
feat: establish graduation transition resolver contract
</commit_message>
<xml_diff>
--- a/棒球人生_三年設計排程_易讀版.xlsx
+++ b/棒球人生_三年設計排程_易讀版.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="R42288999008942cd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="Rfabe7a9b6cb94b8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R81ef74cb883a4b40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="Rb19df4028b2d410b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R85d1c7d91df0472e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R4dd5f81b5d1e47e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="R4ae3431103e84a97"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="Ra7c9ad2c8cbe44db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R5e214c6e22fb46d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R9693d8697d024f99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R44d70bf2cb7148ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R2f033faa7cdc440e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -229,7 +229,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="131">
+  <x:cellXfs count="133">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -548,6 +548,10 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -669,7 +673,7 @@
         <x:color rgb="FFFFFFFF"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FF5B9BD5"/>
         </x:patternFill>
       </x:fill>
@@ -721,9 +725,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1129,12 +1133,12 @@
         <x:v>狀態</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="62" customHeight="1">
+    <x:row r="5" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A5" s="22" t="str">
         <x:v>4.3</x:v>
       </x:c>
       <x:c r="B5" s="23" t="str">
-        <x:v>整理遊戲現在記得哪些事情</x:v>
+        <x:v>Architecture Sprint 4.3：成年職涯網路唯讀契約</x:v>
       </x:c>
       <x:c r="C5" s="68" t="str">
         <x:v>●</x:v>
@@ -1145,18 +1149,19 @@
       <x:c r="G5" s="68" t="str"/>
       <x:c r="H5" s="68" t="str"/>
       <x:c r="I5" s="23" t="str">
-        <x:v>遊戲能清楚記得年級、球季、隊內位置、已發生事件與人物登場狀態。</x:v>
+        <x:v>起始基線：da7fea0｜結案基線：98f1197
+建立可驗證、唯讀的成年棒球職涯網路契約；高中畢業後的成年可能節點已有正式結構，但尚未執行 runtime transition。</x:v>
       </x:c>
       <x:c r="J5" s="24" t="str">
-        <x:v>未開始</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="62" customHeight="1">
+        <x:v>完成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A6" s="25" t="str">
         <x:v>4.4</x:v>
       </x:c>
       <x:c r="B6" s="94" t="str">
-        <x:v>決定高中三年怎麼按照順序前進</x:v>
+        <x:v>Architecture Sprint 4.4：高中畢業入口解析契約</x:v>
       </x:c>
       <x:c r="C6" s="130" t="str">
         <x:v>●</x:v>
@@ -1169,10 +1174,10 @@
       <x:c r="G6" s="130" t="str"/>
       <x:c r="H6" s="130" t="str"/>
       <x:c r="I6" s="94" t="str">
-        <x:v>高一、高二、高三與各球季會在正確時間開始和結束，不會突然跳級。</x:v>
+        <x:v>把合法高中畢業結果唯一對應到既有成年入口；交付解析器、合法與非法狀態測試、唯讀／不變測試及 4.4 架構文件。</x:v>
       </x:c>
       <x:c r="J6" s="26" t="str">
-        <x:v>未開始</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="62" customHeight="1">
@@ -1292,6 +1297,19 @@
       <x:c r="J11" s="29" t="str">
         <x:v>未開始</x:v>
       </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="B12" s="132" t="str">
+        <x:v>註：4.5 以後名稱與內容待 Architecture Sprint 4.4 結案後重新規劃。</x:v>
+      </x:c>
+      <x:c r="C12" s="20"/>
+      <x:c r="D12" s="20"/>
+      <x:c r="E12" s="20"/>
+      <x:c r="F12" s="20"/>
+      <x:c r="G12" s="20"/>
+      <x:c r="H12" s="20"/>
+      <x:c r="I12" s="20"/>
+      <x:c r="J12" s="20"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="86" t="str">
@@ -1450,7 +1468,7 @@
         <x:v>狀態</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="108" customHeight="1">
+    <x:row r="5" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A5" s="22" t="str">
         <x:v>4.3</x:v>
       </x:c>
@@ -1458,25 +1476,27 @@
         <x:v>8月上半</x:v>
       </x:c>
       <x:c r="C5" s="23" t="str">
-        <x:v>遊戲對玩家目前的狀況記得不完整，或同一件事有兩種互相矛盾的紀錄。</x:v>
+        <x:v>高中畢業後有哪些成年職涯節點，哪些只是未來候選？</x:v>
       </x:c>
       <x:c r="D5" s="23" t="str">
-        <x:v>年級、球季、守位、隊內位置、已完成事件與人物登場狀態會保持一致。</x:v>
+        <x:v>建立可驗證、唯讀的成年棒球職涯網路契約；成年可能節點已有正式結構，但不執行 runtime transition。</x:v>
       </x:c>
       <x:c r="E5" s="23" t="str">
-        <x:v>遊玩、重新整理與讀檔後，確認這些資料沒有突然改變或互相矛盾。</x:v>
+        <x:v>確認成年職涯網路可辨識、可稽核且呼叫前後不改變遊戲狀態。</x:v>
       </x:c>
       <x:c r="F5" s="23" t="str">
-        <x:v>文案是否順暢、角色台詞是否好看。</x:v>
+        <x:v>成年正式劇情、執行期轉換與目前路線寫入。</x:v>
       </x:c>
       <x:c r="G5" s="23" t="str">
-        <x:v>Career State Model／狀態單一來源</x:v>
+        <x:v>Architecture Sprint 4.3
+Adult Career Network Readonly Contract
+起始：da7fea0｜結案：98f1197</x:v>
       </x:c>
       <x:c r="H5" s="24" t="str">
-        <x:v>未開始</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="108" customHeight="1">
+        <x:v>完成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A6" s="25" t="str">
         <x:v>4.4</x:v>
       </x:c>
@@ -1484,22 +1504,24 @@
         <x:v>8月下半</x:v>
       </x:c>
       <x:c r="C6" s="94" t="str">
-        <x:v>高中三年的時間可能跳錯，或球季尚未結束就進入下一階段。</x:v>
+        <x:v>高三結束後，既有畢業狀態應如何唯一對應到合法成年職涯入口？</x:v>
       </x:c>
       <x:c r="D6" s="94" t="str">
-        <x:v>高一到高三、各球季與年度結算會按照正常順序發生。</x:v>
+        <x:v>不改變玩家畫面；建立 deterministic Resolver，讓合法畢業結果可被解析為唯一既有成年入口。</x:v>
       </x:c>
       <x:c r="E6" s="94" t="str">
-        <x:v>實際前進時間，確認不會跳級、倒退或在錯誤時間出現高年級事件。</x:v>
+        <x:v>所有合法出口都有唯一入口；非法狀態不 silent fallback；Resolver 不修改 Player 或成年 Contract；既有回歸無破壞。</x:v>
       </x:c>
       <x:c r="F6" s="94" t="str">
-        <x:v>增加新的比賽或人物內容。</x:v>
+        <x:v>成年劇情、UI、存檔欄位、能力平衡與正式 runtime routing。</x:v>
       </x:c>
       <x:c r="G6" s="94" t="str">
-        <x:v>High School Calendar Contract</x:v>
+        <x:v>Graduation Transition Resolver Contract
+交付：Resolver、mapping／invalid／readonly tests、4.4 architecture document
+起始基線：98f1197</x:v>
       </x:c>
       <x:c r="H6" s="26" t="str">
-        <x:v>未開始</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="108" customHeight="1">
@@ -2004,20 +2026,20 @@
         <x:v>在本專案中的白話意思</x:v>
       </x:c>
     </x:row>
-    <x:row r="11" ht="42" customHeight="1">
+    <x:row r="11" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A11" s="25" t="str">
-        <x:v>State Model</x:v>
+        <x:v>Adult Career Network Readonly Contract</x:v>
       </x:c>
       <x:c r="B11" s="26" t="str">
-        <x:v>整理遊戲現在記得哪些事情</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="42" customHeight="1">
+        <x:v>整理高中畢業後已存在的成年節點、入口與重新交會位置，但不推進玩家。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A12" s="25" t="str">
-        <x:v>Calendar Contract</x:v>
+        <x:v>Graduation Transition Resolver Contract</x:v>
       </x:c>
       <x:c r="B12" s="26" t="str">
-        <x:v>決定高中三年按照什麼順序前進</x:v>
+        <x:v>把合法高中畢業結果唯一對應到現有成年入口，但不真正進入下一章。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="42" customHeight="1">

</xml_diff>

<commit_message>
chore: close Architecture Sprint 4.6
</commit_message>
<xml_diff>
--- a/棒球人生_三年設計排程_易讀版.xlsx
+++ b/棒球人生_三年設計排程_易讀版.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="R9823988758ff4f90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="Reed60ffc50524185"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R732b16bd2e3a4ab9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R928ea9e7d3a341c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="Rfea999eb8571478f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R843269939fdf456f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="Ra701c638fc464b62"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="Rd2b9954687fa40d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R3354fc7f07d5466a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R9f9a381f01be4174"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="Re37b669cfbcc4bae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R550b48392af54ae2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -197,9 +197,6 @@
     <x:t xml:space="preserve">4.5</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">4.6</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">第一季結束時，你要親自確認的事情</x:t>
   </x:si>
   <x:si>
@@ -310,9 +307,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">成年劇情、Save Schema、新持久 route state、能力平衡與事件內容。</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">9月下半</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">每四週完成一個可驗收的小階段</x:t>
@@ -1312,8 +1306,8 @@
       </x:c>
     </x:row>
     <x:row r="19" ht="14.399999618530273">
-      <x:c r="A19" s="28" t="s">
-        <x:v>40</x:v>
+      <x:c r="A19" s="28" t="str">
+        <x:v>版本：2026-08-08｜本檔案用於排程追蹤，可直接更新各工作表的「狀態」與「Git基線」欄位。</x:v>
       </x:c>
       <x:c r="B19" s="28" t="s">
         <x:v>40</x:v>
@@ -1499,24 +1493,24 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="49.650001525878906" customHeight="1">
-      <x:c r="A8" s="6" t="s">
-        <x:v>60</x:v>
+      <x:c r="A8" s="6" t="str">
+        <x:v>4.6</x:v>
       </x:c>
       <x:c r="B8" s="2" t="str">
         <x:v>Architecture Sprint 4.6：Adult Transition Runtime Routing Boundary</x:v>
       </x:c>
       <x:c r="C8" s="16"/>
       <x:c r="D8" s="16"/>
-      <x:c r="E8" s="16" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="F8" s="16" t="s">
-        <x:v>53</x:v>
+      <x:c r="E8" s="16" t="str">
+        <x:v>●</x:v>
+      </x:c>
+      <x:c r="F8" s="16" t="str">
+        <x:v>●</x:v>
       </x:c>
       <x:c r="G8" s="16"/>
       <x:c r="H8" s="16"/>
       <x:c r="I8" s="2" t="str">
-        <x:v>起始基線：21bbbc5
+        <x:v>起始基線：21bbbc5｜結案基線：b5a09f9
 核心問題：成年轉換期目前的 route 與 event 應由誰唯一判定？
 主要工作：建立唯讀 Adult Transition Runtime Resolver；讓 CareerSpineContract 成為生涯轉換期 route 與 event 的唯一 topology；移除 Runtime 的 duplicated adult transition route mapping；取消 invalid adult runtime state 的 silent fallback。
 測試級別：Architecture Test Level B+／Readonly Runtime Integration</x:v>
@@ -1527,25 +1521,37 @@
     </x:row>
     <x:row r="9" ht="49.650001525878906" customHeight="1">
       <x:c r="A9" s="6" t="str">
-        <x:v>4.7+</x:v>
+        <x:v>4.7</x:v>
       </x:c>
       <x:c r="B9" s="2" t="str">
-        <x:v>待 Architecture Sprint 4.6 結案後重新規劃</x:v>
+        <x:v>Architecture Sprint 4.7：Adult Transition Progression Boundary</x:v>
       </x:c>
       <x:c r="C9" s="16"/>
       <x:c r="D9" s="16"/>
       <x:c r="E9" s="16"/>
       <x:c r="F9" s="16"/>
-      <x:c r="G9" s="16"/>
+      <x:c r="G9" s="16" t="str">
+        <x:v>●</x:v>
+      </x:c>
       <x:c r="H9" s="16"/>
-      <x:c r="I9" s="2"/>
+      <x:c r="I9" s="2" t="str">
+        <x:v>起始基線：b5a09f9
+核心問題：哪一個合法事件完成後，誰有權修改 transitionStep？
+主要工作：建立 Adult Transition Progression Boundary；由 4.6 Runtime Resolver 驗證 completedEventId，只有目前合法事件才能推進 transitionStep；wrong／repeat／invalid／forced state 全部拒絕且 zero mutation。
+交付：career-transition-progression.js、progression／wrong-event／zero-mutation tests、settlement trigger integration、4.7 architecture document
+測試級別：Architecture Test Level C／Runtime Progression Mutation</x:v>
+      </x:c>
       <x:c r="J9" s="7" t="str">
-        <x:v>待重新規劃</x:v>
+        <x:v>待施工</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="49.650001525878906" customHeight="1">
-      <x:c r="A10" s="6"/>
-      <x:c r="B10" s="2"/>
+      <x:c r="A10" s="6" t="str">
+        <x:v>4.8+</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="str">
+        <x:v>待 Architecture Sprint 4.7 結案後重新規劃</x:v>
+      </x:c>
       <x:c r="C10" s="16"/>
       <x:c r="D10" s="16"/>
       <x:c r="E10" s="16"/>
@@ -1553,7 +1559,9 @@
       <x:c r="G10" s="16"/>
       <x:c r="H10" s="16"/>
       <x:c r="I10" s="2"/>
-      <x:c r="J10" s="7"/>
+      <x:c r="J10" s="7" t="str">
+        <x:v>待重新規劃</x:v>
+      </x:c>
     </x:row>
     <x:row r="11" ht="49.650001525878906" customHeight="1">
       <x:c r="A11" s="8"/>
@@ -1569,7 +1577,7 @@
     </x:row>
     <x:row r="12" ht="28.799999237060547">
       <x:c r="B12" s="25" t="str">
-        <x:v>待 Architecture Sprint 4.6 結案後重新規劃</x:v>
+        <x:v>待 Architecture Sprint 4.7 結案後重新規劃</x:v>
       </x:c>
       <x:c r="C12" s="2"/>
       <x:c r="D12" s="2"/>
@@ -1582,7 +1590,7 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="30" t="s">
-        <x:v>61</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B13" s="30"/>
       <x:c r="C13" s="30"/>
@@ -1596,50 +1604,50 @@
     </x:row>
     <x:row r="14" ht="36.75" customHeight="1">
       <x:c r="A14" s="18" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="B14" s="5" t="s">
         <x:v>62</x:v>
-      </x:c>
-      <x:c r="B14" s="5" t="s">
-        <x:v>63</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="36.75" customHeight="1">
       <x:c r="A15" s="19" t="s">
+        <x:v>63</x:v>
+      </x:c>
+      <x:c r="B15" s="7" t="s">
         <x:v>64</x:v>
-      </x:c>
-      <x:c r="B15" s="7" t="s">
-        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="36.75" customHeight="1">
       <x:c r="A16" s="19" t="s">
+        <x:v>65</x:v>
+      </x:c>
+      <x:c r="B16" s="7" t="s">
         <x:v>66</x:v>
-      </x:c>
-      <x:c r="B16" s="7" t="s">
-        <x:v>67</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="36.75" customHeight="1">
       <x:c r="A17" s="19" t="s">
+        <x:v>67</x:v>
+      </x:c>
+      <x:c r="B17" s="7" t="s">
         <x:v>68</x:v>
-      </x:c>
-      <x:c r="B17" s="7" t="s">
-        <x:v>69</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="36.75" customHeight="1">
       <x:c r="A18" s="20" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B18" s="10" t="s">
         <x:v>70</x:v>
-      </x:c>
-      <x:c r="B18" s="10" t="s">
-        <x:v>71</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="36.75" customHeight="1">
       <x:c r="A19" s="20" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B19" s="10" t="s">
         <x:v>72</x:v>
-      </x:c>
-      <x:c r="B19" s="10" t="s">
-        <x:v>73</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1690,7 +1698,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="29" t="s">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="B1" s="29"/>
       <x:c r="C1" s="29"/>
@@ -1718,19 +1726,19 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="C4" s="21" t="s">
+        <x:v>74</x:v>
+      </x:c>
+      <x:c r="D4" s="21" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="D4" s="21" t="s">
+      <x:c r="E4" s="21" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="E4" s="21" t="s">
+      <x:c r="F4" s="21" t="s">
         <x:v>77</x:v>
       </x:c>
-      <x:c r="F4" s="21" t="s">
+      <x:c r="G4" s="21" t="s">
         <x:v>78</x:v>
-      </x:c>
-      <x:c r="G4" s="21" t="s">
-        <x:v>79</x:v>
       </x:c>
       <x:c r="H4" s="21" t="s">
         <x:v>6</x:v>
@@ -1741,22 +1749,22 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="B5" s="4" t="s">
+        <x:v>79</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="s">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="C5" s="4" t="s">
+      <x:c r="D5" s="4" t="s">
         <x:v>81</x:v>
       </x:c>
-      <x:c r="D5" s="4" t="s">
+      <x:c r="E5" s="4" t="s">
         <x:v>82</x:v>
       </x:c>
-      <x:c r="E5" s="4" t="s">
+      <x:c r="F5" s="4" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="F5" s="4" t="s">
+      <x:c r="G5" s="4" t="s">
         <x:v>84</x:v>
-      </x:c>
-      <x:c r="G5" s="4" t="s">
-        <x:v>85</x:v>
       </x:c>
       <x:c r="H5" s="5" t="s">
         <x:v>55</x:v>
@@ -1767,22 +1775,22 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
+        <x:v>85</x:v>
+      </x:c>
+      <x:c r="C6" s="2" t="s">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="C6" s="2" t="s">
+      <x:c r="D6" s="2" t="s">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="D6" s="2" t="s">
+      <x:c r="E6" s="2" t="s">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="E6" s="2" t="s">
+      <x:c r="F6" s="2" t="s">
         <x:v>89</x:v>
       </x:c>
-      <x:c r="F6" s="2" t="s">
+      <x:c r="G6" s="2" t="s">
         <x:v>90</x:v>
-      </x:c>
-      <x:c r="G6" s="2" t="s">
-        <x:v>91</x:v>
       </x:c>
       <x:c r="H6" s="7" t="s">
         <x:v>55</x:v>
@@ -1793,19 +1801,19 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
+        <x:v>91</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="C7" s="2" t="s">
+      <x:c r="D7" s="2" t="s">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="D7" s="2" t="s">
+      <x:c r="E7" s="2" t="s">
         <x:v>94</x:v>
       </x:c>
-      <x:c r="E7" s="2" t="s">
+      <x:c r="F7" s="2" t="s">
         <x:v>95</x:v>
-      </x:c>
-      <x:c r="F7" s="2" t="s">
-        <x:v>96</x:v>
       </x:c>
       <x:c r="G7" s="2" t="str">
         <x:v>Graduation Transition Commit Boundary
@@ -1817,11 +1825,11 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="86.4000015258789" customHeight="1">
-      <x:c r="A8" s="6" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="B8" s="2" t="s">
-        <x:v>97</x:v>
+      <x:c r="A8" s="6" t="str">
+        <x:v>4.6</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="str">
+        <x:v>9月下半</x:v>
       </x:c>
       <x:c r="C8" s="2" t="str">
         <x:v>成年轉換期目前的 route 與 event 應由誰唯一判定？</x:v>
@@ -1830,15 +1838,14 @@
         <x:v>建立唯讀 Adult Transition Runtime Resolver；讓 CareerSpineContract 成為生涯轉換期 route 與 event 的唯一 topology；移除 Runtime 的 duplicated adult transition route mapping；取消 invalid adult runtime state 的 silent fallback。</x:v>
       </x:c>
       <x:c r="E8" s="2" t="str">
+        <x:v>career-transition-runtime-resolver.js；runtime resolver tests；成年 routing integration tests；legal route/step matrix；invalid-state tests；4.6 architecture document</x:v>
+      </x:c>
+      <x:c r="F8" s="2" t="str">
         <x:v>CareerSpineContract route = Runtime Resolver route = Narrative route = getCurrentEventId() event route。invalid adult runtime state 不得 fallback 到 draft 或 rehab。Resolver 不修改 Player、Save 或 Contract。</x:v>
       </x:c>
-      <x:c r="F8" s="2" t="str">
-        <x:v>成年內容、Save Schema、Progression ownership、能力平衡、事件內容與 UI。</x:v>
-      </x:c>
       <x:c r="G8" s="2" t="str">
-        <x:v>Adult Transition Runtime Routing Boundary
-交付：career-transition-runtime-resolver.js；runtime resolver tests；成年 routing integration tests；legal route/step matrix；invalid-state tests；4.6 architecture document
-起始基線：21bbbc5
+        <x:v>起始基線：21bbbc5
+結案基線：b5a09f9
 Architecture Test Level B+
 Readonly Runtime Integration</x:v>
       </x:c>
@@ -1848,29 +1855,47 @@
     </x:row>
     <x:row r="9" ht="86.4000015258789" customHeight="1">
       <x:c r="A9" s="6" t="str">
-        <x:v>4.7+</x:v>
-      </x:c>
-      <x:c r="B9" s="2"/>
+        <x:v>4.7</x:v>
+      </x:c>
+      <x:c r="B9" s="2" t="str">
+        <x:v>10月上半</x:v>
+      </x:c>
       <x:c r="C9" s="2" t="str">
-        <x:v>待 Architecture Sprint 4.6 結案後重新規劃</x:v>
-      </x:c>
-      <x:c r="D9" s="2"/>
-      <x:c r="E9" s="2"/>
-      <x:c r="F9" s="2"/>
-      <x:c r="G9" s="2"/>
+        <x:v>哪一個合法事件完成後，誰有權修改 transitionStep？</x:v>
+      </x:c>
+      <x:c r="D9" s="2" t="str">
+        <x:v>建立 Adult Transition Progression Boundary；由 4.6 Runtime Resolver 驗證 completedEventId，只有目前合法事件才能推進 transitionStep；wrong／repeat／invalid／forced state 全部拒絕且 zero mutation。</x:v>
+      </x:c>
+      <x:c r="E9" s="2" t="str">
+        <x:v>career-transition-progression.js；Progression Boundary tests；wrong-event／repeat-event／zero-mutation tests；settlement trigger integration；4.7 architecture document</x:v>
+      </x:c>
+      <x:c r="F9" s="2" t="str">
+        <x:v>只有 Runtime Resolver 指定的目前合法事件可以使 transitionStep +1；wrong／repeat／invalid／forced state 全部拒絕且 Player zero mutation；step 4 完成後才要求 settlement；不新增 Player／Save schema。</x:v>
+      </x:c>
+      <x:c r="G9" s="2" t="str">
+        <x:v>起始基線：b5a09f9
+Architecture Test Level C
+Runtime Progression Mutation</x:v>
+      </x:c>
       <x:c r="H9" s="7" t="str">
-        <x:v>待重新規劃</x:v>
+        <x:v>待施工</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="86.4000015258789" customHeight="1">
-      <x:c r="A10" s="8"/>
+      <x:c r="A10" s="8" t="str">
+        <x:v>4.8+</x:v>
+      </x:c>
       <x:c r="B10" s="9"/>
-      <x:c r="C10" s="9"/>
+      <x:c r="C10" s="9" t="str">
+        <x:v>待 Architecture Sprint 4.7 結案後重新規劃</x:v>
+      </x:c>
       <x:c r="D10" s="9"/>
       <x:c r="E10" s="9"/>
       <x:c r="F10" s="9"/>
       <x:c r="G10" s="9"/>
-      <x:c r="H10" s="10"/>
+      <x:c r="H10" s="10" t="str">
+        <x:v>待重新規劃</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1912,7 +1937,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="29" t="s">
-        <x:v>98</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="B1" s="29"/>
       <x:c r="C1" s="29"/>
@@ -1928,87 +1953,87 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="21" t="s">
+        <x:v>97</x:v>
+      </x:c>
+      <x:c r="B4" s="21" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="C4" s="21" t="s">
         <x:v>99</x:v>
       </x:c>
-      <x:c r="B4" s="21" t="s">
+      <x:c r="D4" s="21" t="s">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="C4" s="21" t="s">
+      <x:c r="E4" s="21" t="s">
         <x:v>101</x:v>
-      </x:c>
-      <x:c r="D4" s="21" t="s">
-        <x:v>102</x:v>
-      </x:c>
-      <x:c r="E4" s="21" t="s">
-        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="60.75" customHeight="1">
       <x:c r="A5" s="3" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
+        <x:v>103</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="s">
         <x:v>104</x:v>
       </x:c>
-      <x:c r="B5" s="4" t="s">
+      <x:c r="D5" s="4" t="s">
         <x:v>105</x:v>
       </x:c>
-      <x:c r="C5" s="4" t="s">
+      <x:c r="E5" s="5" t="s">
         <x:v>106</x:v>
-      </x:c>
-      <x:c r="D5" s="4" t="s">
-        <x:v>107</x:v>
-      </x:c>
-      <x:c r="E5" s="5" t="s">
-        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="60.75" customHeight="1">
       <x:c r="A6" s="6" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="B6" s="2" t="s">
+        <x:v>108</x:v>
+      </x:c>
+      <x:c r="C6" s="2" t="s">
         <x:v>109</x:v>
       </x:c>
-      <x:c r="B6" s="2" t="s">
+      <x:c r="D6" s="2" t="s">
         <x:v>110</x:v>
       </x:c>
-      <x:c r="C6" s="2" t="s">
+      <x:c r="E6" s="7" t="s">
         <x:v>111</x:v>
-      </x:c>
-      <x:c r="D6" s="2" t="s">
-        <x:v>112</x:v>
-      </x:c>
-      <x:c r="E6" s="7" t="s">
-        <x:v>113</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="60.75" customHeight="1">
       <x:c r="A7" s="6" t="s">
+        <x:v>112</x:v>
+      </x:c>
+      <x:c r="B7" s="2" t="s">
+        <x:v>113</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="s">
         <x:v>114</x:v>
       </x:c>
-      <x:c r="B7" s="2" t="s">
+      <x:c r="D7" s="2" t="s">
         <x:v>115</x:v>
       </x:c>
-      <x:c r="C7" s="2" t="s">
+      <x:c r="E7" s="7" t="s">
         <x:v>116</x:v>
-      </x:c>
-      <x:c r="D7" s="2" t="s">
-        <x:v>117</x:v>
-      </x:c>
-      <x:c r="E7" s="7" t="s">
-        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="60.75" customHeight="1">
       <x:c r="A8" s="8" t="s">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="B8" s="9" t="s">
+        <x:v>118</x:v>
+      </x:c>
+      <x:c r="C8" s="9" t="s">
         <x:v>119</x:v>
       </x:c>
-      <x:c r="B8" s="9" t="s">
+      <x:c r="D8" s="9" t="s">
         <x:v>120</x:v>
       </x:c>
-      <x:c r="C8" s="9" t="s">
+      <x:c r="E8" s="10" t="s">
         <x:v>121</x:v>
-      </x:c>
-      <x:c r="D8" s="9" t="s">
-        <x:v>122</x:v>
-      </x:c>
-      <x:c r="E8" s="10" t="s">
-        <x:v>123</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2031,7 +2056,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="26" t="s">
-        <x:v>124</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="B1" s="26"/>
       <x:c r="C1" s="26"/>
@@ -2045,114 +2070,114 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="1" t="s">
+        <x:v>123</x:v>
+      </x:c>
+      <x:c r="B4" s="1" t="s">
+        <x:v>124</x:v>
+      </x:c>
+      <x:c r="C4" s="1" t="s">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="B4" s="1" t="s">
+      <x:c r="D4" s="1" t="s">
         <x:v>126</x:v>
-      </x:c>
-      <x:c r="C4" s="1" t="s">
-        <x:v>127</x:v>
-      </x:c>
-      <x:c r="D4" s="1" t="s">
-        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="43.20000076293945" customHeight="1">
       <x:c r="A5" s="3" t="s">
+        <x:v>127</x:v>
+      </x:c>
+      <x:c r="B5" s="4" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="C5" s="4" t="s">
         <x:v>129</x:v>
       </x:c>
-      <x:c r="B5" s="4" t="s">
+      <x:c r="D5" s="5" t="s">
         <x:v>130</x:v>
-      </x:c>
-      <x:c r="C5" s="4" t="s">
-        <x:v>131</x:v>
-      </x:c>
-      <x:c r="D5" s="5" t="s">
-        <x:v>132</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="43.20000076293945" customHeight="1">
       <x:c r="A6" s="6" t="s">
-        <x:v>133</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="C6" s="2" t="s">
+        <x:v>132</x:v>
+      </x:c>
+      <x:c r="D6" s="7" t="s">
         <x:v>130</x:v>
-      </x:c>
-      <x:c r="C6" s="2" t="s">
-        <x:v>134</x:v>
-      </x:c>
-      <x:c r="D6" s="7" t="s">
-        <x:v>132</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="43.20000076293945" customHeight="1">
       <x:c r="A7" s="6" t="s">
-        <x:v>135</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="B7" s="2" t="s">
+        <x:v>128</x:v>
+      </x:c>
+      <x:c r="C7" s="2" t="s">
+        <x:v>134</x:v>
+      </x:c>
+      <x:c r="D7" s="7" t="s">
         <x:v>130</x:v>
-      </x:c>
-      <x:c r="C7" s="2" t="s">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="D7" s="7" t="s">
-        <x:v>132</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="43.20000076293945" customHeight="1">
       <x:c r="A8" s="6" t="s">
+        <x:v>135</x:v>
+      </x:c>
+      <x:c r="B8" s="2" t="s">
+        <x:v>136</x:v>
+      </x:c>
+      <x:c r="C8" s="2" t="s">
         <x:v>137</x:v>
       </x:c>
-      <x:c r="B8" s="2" t="s">
-        <x:v>138</x:v>
-      </x:c>
-      <x:c r="C8" s="2" t="s">
-        <x:v>139</x:v>
-      </x:c>
       <x:c r="D8" s="7" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="43.20000076293945" customHeight="1">
       <x:c r="A9" s="6" t="s">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="B9" s="2" t="s">
+        <x:v>139</x:v>
+      </x:c>
+      <x:c r="C9" s="2" t="s">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="B9" s="2" t="s">
-        <x:v>141</x:v>
-      </x:c>
-      <x:c r="C9" s="2" t="s">
-        <x:v>142</x:v>
-      </x:c>
       <x:c r="D9" s="7" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="43.20000076293945" customHeight="1">
       <x:c r="A10" s="6" t="s">
+        <x:v>141</x:v>
+      </x:c>
+      <x:c r="B10" s="2" t="s">
+        <x:v>142</x:v>
+      </x:c>
+      <x:c r="C10" s="2" t="s">
         <x:v>143</x:v>
       </x:c>
-      <x:c r="B10" s="2" t="s">
-        <x:v>144</x:v>
-      </x:c>
-      <x:c r="C10" s="2" t="s">
-        <x:v>145</x:v>
-      </x:c>
       <x:c r="D10" s="7" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="43.20000076293945" customHeight="1">
       <x:c r="A11" s="8" t="s">
+        <x:v>144</x:v>
+      </x:c>
+      <x:c r="B11" s="9" t="s">
+        <x:v>145</x:v>
+      </x:c>
+      <x:c r="C11" s="9" t="s">
         <x:v>146</x:v>
       </x:c>
-      <x:c r="B11" s="9" t="s">
-        <x:v>147</x:v>
-      </x:c>
-      <x:c r="C11" s="9" t="s">
-        <x:v>148</x:v>
-      </x:c>
       <x:c r="D11" s="10" t="s">
-        <x:v>132</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2191,7 +2216,7 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="29" t="s">
-        <x:v>149</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="B1" s="29"/>
       <x:c r="C1" s="29"/>
@@ -2209,7 +2234,7 @@
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="30" t="s">
-        <x:v>150</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B4" s="30"/>
       <x:c r="C4" s="30"/>
@@ -2219,40 +2244,40 @@
     </x:row>
     <x:row r="5" ht="33.599998474121094" customHeight="1">
       <x:c r="A5" s="18" t="s">
-        <x:v>62</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B5" s="4" t="s">
-        <x:v>151</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>152</x:v>
+        <x:v>150</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="33.599998474121094" customHeight="1">
       <x:c r="A6" s="19" t="s">
-        <x:v>64</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B6" s="2" t="s">
-        <x:v>153</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="C6" s="7" t="s">
-        <x:v>154</x:v>
+        <x:v>152</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="33.599998474121094" customHeight="1">
       <x:c r="A7" s="20" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B7" s="9" t="s">
-        <x:v>155</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="C7" s="10" t="s">
-        <x:v>156</x:v>
+        <x:v>154</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="30" t="s">
-        <x:v>157</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="B9" s="30"/>
       <x:c r="C9" s="30"/>
@@ -2262,63 +2287,63 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="22" t="s">
-        <x:v>158</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="B10" s="23" t="s">
-        <x:v>159</x:v>
+        <x:v>157</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="31.649999618530273" customHeight="1">
       <x:c r="A11" s="6" t="s">
-        <x:v>160</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B11" s="7" t="s">
-        <x:v>161</x:v>
+        <x:v>159</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="31.649999618530273" customHeight="1">
       <x:c r="A12" s="6" t="s">
-        <x:v>162</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="B12" s="7" t="s">
-        <x:v>163</x:v>
+        <x:v>161</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="33.599998474121094" customHeight="1">
       <x:c r="A13" s="6" t="s">
-        <x:v>164</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B13" s="7" t="s">
-        <x:v>165</x:v>
+        <x:v>163</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="33.599998474121094" customHeight="1">
       <x:c r="A14" s="6" t="s">
-        <x:v>166</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B14" s="7" t="s">
-        <x:v>167</x:v>
+        <x:v>165</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="33.599998474121094" customHeight="1">
       <x:c r="A15" s="6" t="s">
-        <x:v>168</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="B15" s="7" t="s">
-        <x:v>169</x:v>
+        <x:v>167</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="33.599998474121094" customHeight="1">
       <x:c r="A16" s="8" t="s">
-        <x:v>170</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B16" s="10" t="s">
-        <x:v>171</x:v>
+        <x:v>169</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="30" t="s">
-        <x:v>172</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B18" s="30"/>
       <x:c r="C18" s="30"/>
@@ -2328,51 +2353,51 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="22" t="s">
+        <x:v>171</x:v>
+      </x:c>
+      <x:c r="B19" s="24" t="s">
+        <x:v>172</x:v>
+      </x:c>
+      <x:c r="C19" s="23" t="s">
         <x:v>173</x:v>
-      </x:c>
-      <x:c r="B19" s="24" t="s">
-        <x:v>174</x:v>
-      </x:c>
-      <x:c r="C19" s="23" t="s">
-        <x:v>175</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="43.20000076293945" customHeight="1">
       <x:c r="A20" s="6" t="s">
+        <x:v>174</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="s">
+        <x:v>175</x:v>
+      </x:c>
+      <x:c r="C20" s="7" t="s">
         <x:v>176</x:v>
-      </x:c>
-      <x:c r="B20" s="2" t="s">
-        <x:v>177</x:v>
-      </x:c>
-      <x:c r="C20" s="7" t="s">
-        <x:v>178</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="43.20000076293945" customHeight="1">
       <x:c r="A21" s="6" t="s">
+        <x:v>177</x:v>
+      </x:c>
+      <x:c r="B21" s="2" t="s">
+        <x:v>178</x:v>
+      </x:c>
+      <x:c r="C21" s="7" t="s">
         <x:v>179</x:v>
-      </x:c>
-      <x:c r="B21" s="2" t="s">
-        <x:v>180</x:v>
-      </x:c>
-      <x:c r="C21" s="7" t="s">
-        <x:v>181</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="43.20000076293945" customHeight="1">
       <x:c r="A22" s="8" t="s">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="B22" s="9" t="s">
+        <x:v>181</x:v>
+      </x:c>
+      <x:c r="C22" s="10" t="s">
         <x:v>182</x:v>
-      </x:c>
-      <x:c r="B22" s="9" t="s">
-        <x:v>183</x:v>
-      </x:c>
-      <x:c r="C22" s="10" t="s">
-        <x:v>184</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="30" t="s">
-        <x:v>185</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="B24" s="30"/>
       <x:c r="C24" s="30"/>
@@ -2382,7 +2407,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="31" t="s">
-        <x:v>186</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="B25" s="32"/>
       <x:c r="C25" s="32"/>

</xml_diff>

<commit_message>
feat: establish adult transition progression boundary
</commit_message>
<xml_diff>
--- a/棒球人生_三年設計排程_易讀版.xlsx
+++ b/棒球人生_三年設計排程_易讀版.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="Ra701c638fc464b62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="Rd2b9954687fa40d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R3354fc7f07d5466a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R9f9a381f01be4174"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="Re37b669cfbcc4bae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R550b48392af54ae2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="Rbc0c5c3f17334b8e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R39ca05316ea34792"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R8c1fca6054464ac2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="Refa04c266f8c4ab0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R1f2aa536ca134eb6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R5aacf5309b0e497c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1535,14 +1535,15 @@
       </x:c>
       <x:c r="H9" s="16"/>
       <x:c r="I9" s="2" t="str">
-        <x:v>起始基線：b5a09f9
+        <x:v>開工 HEAD：9e799a2
+承接技術基線：b5a09f9
 核心問題：哪一個合法事件完成後，誰有權修改 transitionStep？
 主要工作：建立 Adult Transition Progression Boundary；由 4.6 Runtime Resolver 驗證 completedEventId，只有目前合法事件才能推進 transitionStep；wrong／repeat／invalid／forced state 全部拒絕且 zero mutation。
 交付：career-transition-progression.js、progression／wrong-event／zero-mutation tests、settlement trigger integration、4.7 architecture document
 測試級別：Architecture Test Level C／Runtime Progression Mutation</x:v>
       </x:c>
       <x:c r="J9" s="7" t="str">
-        <x:v>待施工</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="49.650001525878906" customHeight="1">
@@ -1873,12 +1874,13 @@
         <x:v>只有 Runtime Resolver 指定的目前合法事件可以使 transitionStep +1；wrong／repeat／invalid／forced state 全部拒絕且 Player zero mutation；step 4 完成後才要求 settlement；不新增 Player／Save schema。</x:v>
       </x:c>
       <x:c r="G9" s="2" t="str">
-        <x:v>起始基線：b5a09f9
+        <x:v>開工 HEAD：9e799a2
+承接技術基線：b5a09f9
 Architecture Test Level C
 Runtime Progression Mutation</x:v>
       </x:c>
       <x:c r="H9" s="7" t="str">
-        <x:v>待施工</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="86.4000015258789" customHeight="1">

</xml_diff>

<commit_message>
feat: establish development years runtime routing boundary
</commit_message>
<xml_diff>
--- a/棒球人生_三年設計排程_易讀版.xlsx
+++ b/棒球人生_三年設計排程_易讀版.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="Rbc0c5c3f17334b8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R39ca05316ea34792"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R8c1fca6054464ac2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="Refa04c266f8c4ab0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R1f2aa536ca134eb6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R5aacf5309b0e497c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="Ra4f033d8eb7044a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="Rf6b675603c53425c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R0b10d89d7b294831"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="Rd488e6fba66f4095"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R8d700f297c6641cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R61af0bd5ce214d34"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1535,11 +1535,9 @@
       </x:c>
       <x:c r="H9" s="16"/>
       <x:c r="I9" s="2" t="str">
-        <x:v>開工 HEAD：9e799a2
-承接技術基線：b5a09f9
+        <x:v>開工 HEAD：9e799a2｜承接技術基線：b5a09f9｜結案基線：78e65e3
 核心問題：哪一個合法事件完成後，誰有權修改 transitionStep？
-主要工作：建立 Adult Transition Progression Boundary；由 4.6 Runtime Resolver 驗證 completedEventId，只有目前合法事件才能推進 transitionStep；wrong／repeat／invalid／forced state 全部拒絕且 zero mutation。
-交付：career-transition-progression.js、progression／wrong-event／zero-mutation tests、settlement trigger integration、4.7 architecture document
+主要成果：建立 Adult Transition Progression Boundary；由 4.6 Runtime Resolver 驗證 completedEventId；只有目前合法事件才能推進 transitionStep；wrong／repeat／invalid／forced state 全部拒絕且 zero mutation；terminal settlement exactly once。
 測試級別：Architecture Test Level C／Runtime Progression Mutation</x:v>
       </x:c>
       <x:c r="J9" s="7" t="str">
@@ -1548,25 +1546,37 @@
     </x:row>
     <x:row r="10" ht="49.650001525878906" customHeight="1">
       <x:c r="A10" s="6" t="str">
-        <x:v>4.8+</x:v>
+        <x:v>4.8</x:v>
       </x:c>
       <x:c r="B10" s="2" t="str">
-        <x:v>待 Architecture Sprint 4.7 結案後重新規劃</x:v>
+        <x:v>Architecture Sprint 4.8：Development Years Runtime Routing Boundary</x:v>
       </x:c>
       <x:c r="C10" s="16"/>
       <x:c r="D10" s="16"/>
       <x:c r="E10" s="16"/>
       <x:c r="F10" s="16"/>
       <x:c r="G10" s="16"/>
-      <x:c r="H10" s="16"/>
-      <x:c r="I10" s="2"/>
+      <x:c r="H10" s="16" t="str">
+        <x:v>●</x:v>
+      </x:c>
+      <x:c r="I10" s="2" t="str">
+        <x:v>起始基線：78e65e3
+核心問題：20–21 歲發展期（通往 22 歲職涯小結）的 route 與 current event 應由誰唯一判定？
+主要工作：建立唯讀 Development Years Runtime Resolver；以 CareerSpineContract 的正式 careerExit mapping 與 sharedDevelopment.eventIds 作為唯一 topology；移除 story.js duplicated development sequence；取消 invalid careerExit／developmentStep 的 silent fallback。
+Legal Matrix：5 careerExit × 7 developmentStep = 35 cases
+測試級別：Architecture Test Level B+／Readonly Development Runtime Integration</x:v>
+      </x:c>
       <x:c r="J10" s="7" t="str">
-        <x:v>待重新規劃</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="49.650001525878906" customHeight="1">
-      <x:c r="A11" s="8"/>
-      <x:c r="B11" s="9"/>
+      <x:c r="A11" s="8" t="str">
+        <x:v>4.9+</x:v>
+      </x:c>
+      <x:c r="B11" s="9" t="str">
+        <x:v>待 Architecture Sprint 4.8 結案後重新規劃</x:v>
+      </x:c>
       <x:c r="C11" s="17"/>
       <x:c r="D11" s="17"/>
       <x:c r="E11" s="17"/>
@@ -1574,11 +1584,13 @@
       <x:c r="G11" s="17"/>
       <x:c r="H11" s="17"/>
       <x:c r="I11" s="9"/>
-      <x:c r="J11" s="10"/>
+      <x:c r="J11" s="10" t="str">
+        <x:v>待重新規劃</x:v>
+      </x:c>
     </x:row>
     <x:row r="12" ht="28.799999237060547">
       <x:c r="B12" s="25" t="str">
-        <x:v>待 Architecture Sprint 4.7 結案後重新規劃</x:v>
+        <x:v>待 Architecture Sprint 4.8 結案後重新規劃</x:v>
       </x:c>
       <x:c r="C12" s="2"/>
       <x:c r="D12" s="2"/>
@@ -1865,17 +1877,18 @@
         <x:v>哪一個合法事件完成後，誰有權修改 transitionStep？</x:v>
       </x:c>
       <x:c r="D9" s="2" t="str">
-        <x:v>建立 Adult Transition Progression Boundary；由 4.6 Runtime Resolver 驗證 completedEventId，只有目前合法事件才能推進 transitionStep；wrong／repeat／invalid／forced state 全部拒絕且 zero mutation。</x:v>
+        <x:v>建立 Adult Transition Progression Boundary；由 4.6 Runtime Resolver 驗證 completedEventId；只有目前合法事件才能推進 transitionStep；wrong／repeat／invalid／forced state 全部拒絕且 zero mutation。</x:v>
       </x:c>
       <x:c r="E9" s="2" t="str">
         <x:v>career-transition-progression.js；Progression Boundary tests；wrong-event／repeat-event／zero-mutation tests；settlement trigger integration；4.7 architecture document</x:v>
       </x:c>
       <x:c r="F9" s="2" t="str">
-        <x:v>只有 Runtime Resolver 指定的目前合法事件可以使 transitionStep +1；wrong／repeat／invalid／forced state 全部拒絕且 Player zero mutation；step 4 完成後才要求 settlement；不新增 Player／Save schema。</x:v>
+        <x:v>只有 Runtime Resolver 指定的目前合法事件可以使 transitionStep +1；wrong／repeat／invalid／forced state 全部拒絕且 Player zero mutation；terminal settlement exactly once；不新增 Player／Save schema。</x:v>
       </x:c>
       <x:c r="G9" s="2" t="str">
         <x:v>開工 HEAD：9e799a2
 承接技術基線：b5a09f9
+結案基線：78e65e3
 Architecture Test Level C
 Runtime Progression Mutation</x:v>
       </x:c>
@@ -1885,17 +1898,45 @@
     </x:row>
     <x:row r="10" ht="86.4000015258789" customHeight="1">
       <x:c r="A10" s="8" t="str">
-        <x:v>4.8+</x:v>
-      </x:c>
-      <x:c r="B10" s="9"/>
+        <x:v>4.8</x:v>
+      </x:c>
+      <x:c r="B10" s="9" t="str">
+        <x:v>10月下半</x:v>
+      </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>待 Architecture Sprint 4.7 結案後重新規劃</x:v>
-      </x:c>
-      <x:c r="D10" s="9"/>
-      <x:c r="E10" s="9"/>
-      <x:c r="F10" s="9"/>
-      <x:c r="G10" s="9"/>
+        <x:v>20–21 歲發展期（通往 22 歲職涯小結）的 route 與 current event 應由誰唯一判定？</x:v>
+      </x:c>
+      <x:c r="D10" s="9" t="str">
+        <x:v>建立唯讀 Development Years Runtime Resolver；以 CareerSpineContract 的正式 careerExit mapping 與 sharedDevelopment.eventIds 作為唯一 topology；移除 story.js duplicated development sequence；取消 invalid careerExit／developmentStep 的 silent fallback。</x:v>
+      </x:c>
+      <x:c r="E10" s="9" t="str">
+        <x:v>career-development-runtime-resolver.js；Development Runtime Resolver tests；35-case legal matrix；invalid-state tests；runtime／Narrative invariant tests；4.8 architecture document</x:v>
+      </x:c>
+      <x:c r="F10" s="9" t="str">
+        <x:v>5 個 careerExit × 7 個合法 developmentStep 全部解析正確；Contract route = Development Resolver route = Narrative route；Contract sharedDevelopment event = Resolver event = getCurrentEventId()；invalid careerExit／step／wrong chapter 一律 unresolved，不 fallback 到 draft 或 development_result；Resolver 不修改 Player、Save 或 Contract。</x:v>
+      </x:c>
+      <x:c r="G10" s="9" t="str">
+        <x:v>起始基線：78e65e3
+Architecture Test Level B+
+Readonly Development Runtime Integration</x:v>
+      </x:c>
       <x:c r="H10" s="10" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>4.9+</x:v>
+      </x:c>
+      <x:c r="B11"/>
+      <x:c r="C11" t="str">
+        <x:v>待 Architecture Sprint 4.8 結案後重新規劃</x:v>
+      </x:c>
+      <x:c r="D11"/>
+      <x:c r="E11"/>
+      <x:c r="F11"/>
+      <x:c r="G11"/>
+      <x:c r="H11" t="str">
         <x:v>待重新規劃</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat: establish development years progression boundary
</commit_message>
<xml_diff>
--- a/棒球人生_三年設計排程_易讀版.xlsx
+++ b/棒球人生_三年設計排程_易讀版.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="Ra4f033d8eb7044a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="Rf6b675603c53425c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R0b10d89d7b294831"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="Rd488e6fba66f4095"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R8d700f297c6641cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R61af0bd5ce214d34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="R138e4b1ff2f84cf0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R2cff1401266c4c0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R8f188ea3d4134b8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="Rf0bf2a4d00cd4095"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R3e7d7dc467214c0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R4ddb9eee7ad04dfb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1560,9 +1560,9 @@
         <x:v>●</x:v>
       </x:c>
       <x:c r="I10" s="2" t="str">
-        <x:v>起始基線：78e65e3
+        <x:v>起始基線：78e65e3｜結案基線：2aacf0d
 核心問題：20–21 歲發展期（通往 22 歲職涯小結）的 route 與 current event 應由誰唯一判定？
-主要工作：建立唯讀 Development Years Runtime Resolver；以 CareerSpineContract 的正式 careerExit mapping 與 sharedDevelopment.eventIds 作為唯一 topology；移除 story.js duplicated development sequence；取消 invalid careerExit／developmentStep 的 silent fallback。
+主要成果：建立唯讀 Development Years Runtime Resolver；以 CareerSpineContract 的正式 careerExit mapping 與 sharedDevelopment.eventIds 作為唯一 topology；移除 story.js／script.js duplicated development topology；取消 invalid careerExit／developmentStep 的 silent fallback。
 Legal Matrix：5 careerExit × 7 developmentStep = 35 cases
 測試級別：Architecture Test Level B+／Readonly Development Runtime Integration</x:v>
       </x:c>
@@ -1572,10 +1572,10 @@
     </x:row>
     <x:row r="11" ht="49.650001525878906" customHeight="1">
       <x:c r="A11" s="8" t="str">
-        <x:v>4.9+</x:v>
+        <x:v>4.9</x:v>
       </x:c>
       <x:c r="B11" s="9" t="str">
-        <x:v>待 Architecture Sprint 4.8 結案後重新規劃</x:v>
+        <x:v>Architecture Sprint 4.9：Development Years Progression Boundary</x:v>
       </x:c>
       <x:c r="C11" s="17"/>
       <x:c r="D11" s="17"/>
@@ -1583,14 +1583,24 @@
       <x:c r="F11" s="17"/>
       <x:c r="G11" s="17"/>
       <x:c r="H11" s="17"/>
-      <x:c r="I11" s="9"/>
+      <x:c r="I11" s="9" t="str">
+        <x:v>起始基線：2aacf0d
+核心問題：只有真正完成目前合法 Development event 的玩家，誰有權讓 developmentStep 往下一格？
+主要工作：建立 Development Years Progression Boundary；由 4.8 Runtime Resolver 驗證 completedEventId；正常 Gameplay 的 developmentStep +1 改由唯一 Boundary 授權；發展期 stale／wrong／repeat／forced event 在 effects 前拒絕；最後一幕只允許觸發一次 22 歲結算。
+Legal Matrix：5 careerExit × 7 developmentStep = 35 progression cases
+測試級別：Architecture Test Level C／Runtime Development Progression Mutation
+排程：第一季追加 Sprint（不虛構既有甘特圖之外的日期）</x:v>
+      </x:c>
       <x:c r="J11" s="10" t="str">
-        <x:v>待重新規劃</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="28.799999237060547">
+      <x:c r="A12" t="str">
+        <x:v>4.10+</x:v>
+      </x:c>
       <x:c r="B12" s="25" t="str">
-        <x:v>待 Architecture Sprint 4.8 結案後重新規劃</x:v>
+        <x:v>待 Architecture Sprint 4.9 結案後重新規劃</x:v>
       </x:c>
       <x:c r="C12" s="2"/>
       <x:c r="D12" s="2"/>
@@ -1599,7 +1609,9 @@
       <x:c r="G12" s="2"/>
       <x:c r="H12" s="2"/>
       <x:c r="I12" s="2"/>
-      <x:c r="J12" s="2"/>
+      <x:c r="J12" s="2" t="str">
+        <x:v>待重新規劃</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="30" t="s">
@@ -1907,16 +1919,17 @@
         <x:v>20–21 歲發展期（通往 22 歲職涯小結）的 route 與 current event 應由誰唯一判定？</x:v>
       </x:c>
       <x:c r="D10" s="9" t="str">
-        <x:v>建立唯讀 Development Years Runtime Resolver；以 CareerSpineContract 的正式 careerExit mapping 與 sharedDevelopment.eventIds 作為唯一 topology；移除 story.js duplicated development sequence；取消 invalid careerExit／developmentStep 的 silent fallback。</x:v>
+        <x:v>建立唯讀 Development Years Runtime Resolver；以 CareerSpineContract 的正式 careerExit mapping 與 sharedDevelopment.eventIds 作為唯一 topology；移除 duplicated development topology；取消 invalid careerExit／developmentStep 的 silent fallback。</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
         <x:v>career-development-runtime-resolver.js；Development Runtime Resolver tests；35-case legal matrix；invalid-state tests；runtime／Narrative invariant tests；4.8 architecture document</x:v>
       </x:c>
       <x:c r="F10" s="9" t="str">
-        <x:v>5 個 careerExit × 7 個合法 developmentStep 全部解析正確；Contract route = Development Resolver route = Narrative route；Contract sharedDevelopment event = Resolver event = getCurrentEventId()；invalid careerExit／step／wrong chapter 一律 unresolved，不 fallback 到 draft 或 development_result；Resolver 不修改 Player、Save 或 Contract。</x:v>
+        <x:v>5 個 careerExit × 7 個合法 developmentStep 全部解析正確；Contract route = Development Resolver route = Narrative route；Contract sharedDevelopment event = Resolver event = getCurrentEventId()；invalid careerExit／step／wrong chapter 一律 unresolved；Resolver 不修改 Player、Save 或 Contract。</x:v>
       </x:c>
       <x:c r="G10" s="9" t="str">
         <x:v>起始基線：78e65e3
+結案基線：2aacf0d
 Architecture Test Level B+
 Readonly Development Runtime Integration</x:v>
       </x:c>
@@ -1926,17 +1939,45 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>4.9+</x:v>
-      </x:c>
-      <x:c r="B11"/>
+        <x:v>4.9</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>第一季追加</x:v>
+      </x:c>
       <x:c r="C11" t="str">
-        <x:v>待 Architecture Sprint 4.8 結案後重新規劃</x:v>
-      </x:c>
-      <x:c r="D11"/>
-      <x:c r="E11"/>
-      <x:c r="F11"/>
-      <x:c r="G11"/>
+        <x:v>只有真正完成目前合法 Development event 的玩家，誰有權讓 developmentStep 往下一格？</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>建立 Development Years Progression Boundary；由 4.8 Runtime Resolver 驗證 completedEventId；正常 Gameplay 的 developmentStep +1 改由唯一 Boundary 授權；發展期 stale／wrong／repeat／forced event 在 effects 前拒絕。</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>career-development-progression.js；Progression Boundary tests；35-case legal progression matrix；wrong／repeat／forced／zero-mutation tests；writable safety；terminal settlement exactly-once integration；4.9 architecture document</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>只有 4.8 Runtime Resolver 指定的目前合法 Development event 可以使 developmentStep +1；wrong／repeat／invalid／forced state 全部拒絕且 Player zero mutation；step 6 完成後才要求 settlement，22 歲結算 exactly once；不新增 Player／Save schema。</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>起始基線：2aacf0d
+Architecture Test Level C
+Runtime Development Progression Mutation</x:v>
+      </x:c>
       <x:c r="H11" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" t="str">
+        <x:v>4.10+</x:v>
+      </x:c>
+      <x:c r="B12"/>
+      <x:c r="C12" t="str">
+        <x:v>待 Architecture Sprint 4.9 結案後重新規劃</x:v>
+      </x:c>
+      <x:c r="D12"/>
+      <x:c r="E12"/>
+      <x:c r="F12"/>
+      <x:c r="G12"/>
+      <x:c r="H12" t="str">
         <x:v>待重新規劃</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
feat: establish adult career save admission boundary
</commit_message>
<xml_diff>
--- a/棒球人生_三年設計排程_易讀版.xlsx
+++ b/棒球人生_三年設計排程_易讀版.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="R138e4b1ff2f84cf0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R2cff1401266c4c0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R8f188ea3d4134b8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="Rf0bf2a4d00cd4095"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R3e7d7dc467214c0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R4ddb9eee7ad04dfb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="R5b0218c1d7174dbf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R52c36708a5484917"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="Rc34b980a347e4a0f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R120101270eda430b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R5983230362ca427c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R30e6520caf3e43fa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1356,7 +1356,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="13.800000190734863"/>
   <x:cols>
-    <x:col min="1" max="1" width="10" customWidth="1"/>
+    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="34" customWidth="1"/>
     <x:col min="3" max="8" width="13" customWidth="1"/>
     <x:col min="9" max="9" width="48" customWidth="1"/>
@@ -1584,12 +1584,12 @@
       <x:c r="G11" s="17"/>
       <x:c r="H11" s="17"/>
       <x:c r="I11" s="9" t="str">
-        <x:v>起始基線：2aacf0d
+        <x:v>起始基線：2aacf0d｜結案基線：23f3487
 核心問題：只有真正完成目前合法 Development event 的玩家，誰有權讓 developmentStep 往下一格？
-主要工作：建立 Development Years Progression Boundary；由 4.8 Runtime Resolver 驗證 completedEventId；正常 Gameplay 的 developmentStep +1 改由唯一 Boundary 授權；發展期 stale／wrong／repeat／forced event 在 effects 前拒絕；最後一幕只允許觸發一次 22 歲結算。
+主要成果：建立 Development Years Progression Boundary；由 4.8 Runtime Resolver 驗證 completedEventId；正常 Gameplay 的 developmentStep +1 改由唯一 Boundary 授權；發展期 stale／wrong／repeat／forced event 在 effects 前拒絕；最後一幕只允許觸發一次 22 歲結算。
 Legal Matrix：5 careerExit × 7 developmentStep = 35 progression cases
 測試級別：Architecture Test Level C／Runtime Development Progression Mutation
-排程：第一季追加 Sprint（不虛構既有甘特圖之外的日期）</x:v>
+排程：第一季追加 Sprint</x:v>
       </x:c>
       <x:c r="J11" s="10" t="str">
         <x:v>完成</x:v>
@@ -1597,10 +1597,10 @@
     </x:row>
     <x:row r="12" ht="28.799999237060547">
       <x:c r="A12" t="str">
-        <x:v>4.10+</x:v>
+        <x:v>4.10</x:v>
       </x:c>
       <x:c r="B12" s="25" t="str">
-        <x:v>待 Architecture Sprint 4.9 結案後重新規劃</x:v>
+        <x:v>Architecture Sprint 4.10：Adult Career Save Admission Boundary</x:v>
       </x:c>
       <x:c r="C12" s="2"/>
       <x:c r="D12" s="2"/>
@@ -1608,16 +1608,24 @@
       <x:c r="F12" s="2"/>
       <x:c r="G12" s="2"/>
       <x:c r="H12" s="2"/>
-      <x:c r="I12" s="2"/>
+      <x:c r="I12" s="2" t="str">
+        <x:v>起始基線：23f3487
+核心問題：一份 normalized 成年存檔在成為 live Player 前，誰負責證明它描述的是合法的 18–22 歲職涯位置？
+主要工作：建立 Adult Career Save Admission Boundary；以 CareerSpineContract 為主要狀態權威，並在生涯轉換期／發展期重用既有 Runtime Resolver；loadGame 先 normalize candidate，再 admission，只有 admitted 才能原子替換 live player。非法成年存檔拒絕載入且 live Player／主要 UI 不被污染，不自動修復、不自動刪除。
+測試級別：Architecture Test Level C／Adult Career Save Admission Integration
+排程：第一季追加 Sprint II</x:v>
+      </x:c>
       <x:c r="J12" s="2" t="str">
-        <x:v>待重新規劃</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="30" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="B13" s="30"/>
+      <x:c r="A13" s="30" t="str">
+        <x:v>4.11+</x:v>
+      </x:c>
+      <x:c r="B13" s="30" t="str">
+        <x:v>待 Architecture Sprint 4.10 結案後重新規劃</x:v>
+      </x:c>
       <x:c r="C13" s="30"/>
       <x:c r="D13" s="30"/>
       <x:c r="E13" s="30"/>
@@ -1625,55 +1633,371 @@
       <x:c r="G13" s="30"/>
       <x:c r="H13" s="30"/>
       <x:c r="I13" s="30"/>
-      <x:c r="J13" s="30"/>
+      <x:c r="J13" s="30" t="str">
+        <x:v>待重新規劃</x:v>
+      </x:c>
     </x:row>
     <x:row r="14" ht="36.75" customHeight="1">
       <x:c r="A14" s="18" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="B14" s="5" t="s">
-        <x:v>62</x:v>
-      </x:c>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B14" s="5"/>
+      <x:c r="C14"/>
+      <x:c r="D14"/>
+      <x:c r="E14"/>
+      <x:c r="F14"/>
+      <x:c r="G14"/>
+      <x:c r="H14"/>
+      <x:c r="I14"/>
+      <x:c r="J14"/>
     </x:row>
     <x:row r="15" ht="36.75" customHeight="1">
       <x:c r="A15" s="19" t="s">
-        <x:v>63</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B15" s="7" t="s">
-        <x:v>64</x:v>
-      </x:c>
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="C15"/>
+      <x:c r="D15"/>
+      <x:c r="E15"/>
+      <x:c r="F15"/>
+      <x:c r="G15"/>
+      <x:c r="H15"/>
+      <x:c r="I15"/>
+      <x:c r="J15"/>
     </x:row>
     <x:row r="16" ht="36.75" customHeight="1">
       <x:c r="A16" s="19" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B16" s="7" t="s">
-        <x:v>66</x:v>
-      </x:c>
+        <x:v>64</x:v>
+      </x:c>
+      <x:c r="C16"/>
+      <x:c r="D16"/>
+      <x:c r="E16"/>
+      <x:c r="F16"/>
+      <x:c r="G16"/>
+      <x:c r="H16"/>
+      <x:c r="I16"/>
+      <x:c r="J16"/>
     </x:row>
     <x:row r="17" ht="36.75" customHeight="1">
       <x:c r="A17" s="19" t="s">
-        <x:v>67</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B17" s="7" t="s">
-        <x:v>68</x:v>
-      </x:c>
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="C17"/>
+      <x:c r="D17"/>
+      <x:c r="E17"/>
+      <x:c r="F17"/>
+      <x:c r="G17"/>
+      <x:c r="H17"/>
+      <x:c r="I17"/>
+      <x:c r="J17"/>
     </x:row>
     <x:row r="18" ht="36.75" customHeight="1">
       <x:c r="A18" s="20" t="s">
-        <x:v>69</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B18" s="10" t="s">
-        <x:v>70</x:v>
-      </x:c>
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
+      <x:c r="E18"/>
+      <x:c r="F18"/>
+      <x:c r="G18"/>
+      <x:c r="H18"/>
+      <x:c r="I18"/>
+      <x:c r="J18"/>
     </x:row>
     <x:row r="19" ht="36.75" customHeight="1">
       <x:c r="A19" s="20" t="s">
+        <x:v>69</x:v>
+      </x:c>
+      <x:c r="B19" s="10" t="s">
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
+      <x:c r="E19"/>
+      <x:c r="F19"/>
+      <x:c r="G19"/>
+      <x:c r="H19"/>
+      <x:c r="I19"/>
+      <x:c r="J19"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="B19" s="10" t="s">
+      <x:c r="B20" t="s">
         <x:v>72</x:v>
       </x:c>
+      <x:c r="C20"/>
+      <x:c r="D20"/>
+      <x:c r="E20"/>
+      <x:c r="F20"/>
+      <x:c r="G20"/>
+      <x:c r="H20"/>
+      <x:c r="I20"/>
+      <x:c r="J20"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
+      <x:c r="G21"/>
+      <x:c r="H21"/>
+      <x:c r="I21"/>
+      <x:c r="J21"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22"/>
+      <x:c r="B22"/>
+      <x:c r="C22"/>
+      <x:c r="D22"/>
+      <x:c r="E22"/>
+      <x:c r="F22"/>
+      <x:c r="G22"/>
+      <x:c r="H22"/>
+      <x:c r="I22"/>
+      <x:c r="J22"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23"/>
+      <x:c r="B23"/>
+      <x:c r="C23"/>
+      <x:c r="D23"/>
+      <x:c r="E23"/>
+      <x:c r="F23"/>
+      <x:c r="G23"/>
+      <x:c r="H23"/>
+      <x:c r="I23"/>
+      <x:c r="J23"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24"/>
+      <x:c r="B24"/>
+      <x:c r="C24"/>
+      <x:c r="D24"/>
+      <x:c r="E24"/>
+      <x:c r="F24"/>
+      <x:c r="G24"/>
+      <x:c r="H24"/>
+      <x:c r="I24"/>
+      <x:c r="J24"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25"/>
+      <x:c r="B25"/>
+      <x:c r="C25"/>
+      <x:c r="D25"/>
+      <x:c r="E25"/>
+      <x:c r="F25"/>
+      <x:c r="G25"/>
+      <x:c r="H25"/>
+      <x:c r="I25"/>
+      <x:c r="J25"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26"/>
+      <x:c r="B26"/>
+      <x:c r="C26"/>
+      <x:c r="D26"/>
+      <x:c r="E26"/>
+      <x:c r="F26"/>
+      <x:c r="G26"/>
+      <x:c r="H26"/>
+      <x:c r="I26"/>
+      <x:c r="J26"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27"/>
+      <x:c r="B27"/>
+      <x:c r="C27"/>
+      <x:c r="D27"/>
+      <x:c r="E27"/>
+      <x:c r="F27"/>
+      <x:c r="G27"/>
+      <x:c r="H27"/>
+      <x:c r="I27"/>
+      <x:c r="J27"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28"/>
+      <x:c r="B28"/>
+      <x:c r="C28"/>
+      <x:c r="D28"/>
+      <x:c r="E28"/>
+      <x:c r="F28"/>
+      <x:c r="G28"/>
+      <x:c r="H28"/>
+      <x:c r="I28"/>
+      <x:c r="J28"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29"/>
+      <x:c r="B29"/>
+      <x:c r="C29"/>
+      <x:c r="D29"/>
+      <x:c r="E29"/>
+      <x:c r="F29"/>
+      <x:c r="G29"/>
+      <x:c r="H29"/>
+      <x:c r="I29"/>
+      <x:c r="J29"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30"/>
+      <x:c r="B30"/>
+      <x:c r="C30"/>
+      <x:c r="D30"/>
+      <x:c r="E30"/>
+      <x:c r="F30"/>
+      <x:c r="G30"/>
+      <x:c r="H30"/>
+      <x:c r="I30"/>
+      <x:c r="J30"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31"/>
+      <x:c r="B31"/>
+      <x:c r="C31"/>
+      <x:c r="D31"/>
+      <x:c r="E31"/>
+      <x:c r="F31"/>
+      <x:c r="G31"/>
+      <x:c r="H31"/>
+      <x:c r="I31"/>
+      <x:c r="J31"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32"/>
+      <x:c r="B32"/>
+      <x:c r="C32"/>
+      <x:c r="D32"/>
+      <x:c r="E32"/>
+      <x:c r="F32"/>
+      <x:c r="G32"/>
+      <x:c r="H32"/>
+      <x:c r="I32"/>
+      <x:c r="J32"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33"/>
+      <x:c r="B33"/>
+      <x:c r="C33"/>
+      <x:c r="D33"/>
+      <x:c r="E33"/>
+      <x:c r="F33"/>
+      <x:c r="G33"/>
+      <x:c r="H33"/>
+      <x:c r="I33"/>
+      <x:c r="J33"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34"/>
+      <x:c r="B34"/>
+      <x:c r="C34"/>
+      <x:c r="D34"/>
+      <x:c r="E34"/>
+      <x:c r="F34"/>
+      <x:c r="G34"/>
+      <x:c r="H34"/>
+      <x:c r="I34"/>
+      <x:c r="J34"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35"/>
+      <x:c r="B35"/>
+      <x:c r="C35"/>
+      <x:c r="D35"/>
+      <x:c r="E35"/>
+      <x:c r="F35"/>
+      <x:c r="G35"/>
+      <x:c r="H35"/>
+      <x:c r="I35"/>
+      <x:c r="J35"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36"/>
+      <x:c r="B36"/>
+      <x:c r="C36"/>
+      <x:c r="D36"/>
+      <x:c r="E36"/>
+      <x:c r="F36"/>
+      <x:c r="G36"/>
+      <x:c r="H36"/>
+      <x:c r="I36"/>
+      <x:c r="J36"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37"/>
+      <x:c r="B37"/>
+      <x:c r="C37"/>
+      <x:c r="D37"/>
+      <x:c r="E37"/>
+      <x:c r="F37"/>
+      <x:c r="G37"/>
+      <x:c r="H37"/>
+      <x:c r="I37"/>
+      <x:c r="J37"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38"/>
+      <x:c r="B38"/>
+      <x:c r="C38"/>
+      <x:c r="D38"/>
+      <x:c r="E38"/>
+      <x:c r="F38"/>
+      <x:c r="G38"/>
+      <x:c r="H38"/>
+      <x:c r="I38"/>
+      <x:c r="J38"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39"/>
+      <x:c r="B39"/>
+      <x:c r="C39"/>
+      <x:c r="D39"/>
+      <x:c r="E39"/>
+      <x:c r="F39"/>
+      <x:c r="G39"/>
+      <x:c r="H39"/>
+      <x:c r="I39"/>
+      <x:c r="J39"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40"/>
+      <x:c r="B40"/>
+      <x:c r="C40"/>
+      <x:c r="D40"/>
+      <x:c r="E40"/>
+      <x:c r="F40"/>
+      <x:c r="G40"/>
+      <x:c r="H40"/>
+      <x:c r="I40"/>
+      <x:c r="J40"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41"/>
+      <x:c r="B41"/>
+      <x:c r="C41"/>
+      <x:c r="D41"/>
+      <x:c r="E41"/>
+      <x:c r="F41"/>
+      <x:c r="G41"/>
+      <x:c r="H41"/>
+      <x:c r="I41"/>
+      <x:c r="J41"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1712,7 +2036,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="13.800000190734863"/>
   <x:cols>
-    <x:col min="1" max="1" width="9" customWidth="1"/>
+    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="13" customWidth="1"/>
     <x:col min="3" max="4" width="38" customWidth="1"/>
     <x:col min="5" max="5" width="42" customWidth="1"/>
@@ -1958,6 +2282,7 @@
       </x:c>
       <x:c r="G11" t="str">
         <x:v>起始基線：2aacf0d
+結案基線：23f3487
 Architecture Test Level C
 Runtime Development Progression Mutation</x:v>
       </x:c>
@@ -1967,19 +2292,327 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>4.10+</x:v>
-      </x:c>
-      <x:c r="B12"/>
+        <x:v>4.10</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>第一季追加 II</x:v>
+      </x:c>
       <x:c r="C12" t="str">
-        <x:v>待 Architecture Sprint 4.9 結案後重新規劃</x:v>
-      </x:c>
-      <x:c r="D12"/>
-      <x:c r="E12"/>
-      <x:c r="F12"/>
-      <x:c r="G12"/>
+        <x:v>一份 normalized 成年存檔在成為 live Player 前，誰負責證明它描述的是合法的 18–22 歲職涯位置？</x:v>
+      </x:c>
+      <x:c r="D12" t="str">
+        <x:v>建立 Adult Career Save Admission Boundary；在 normalizeSave() 之後、live player replacement 之前驗證成年 Career state。主要依據 CareerSpineContract；生涯轉換期與發展期再重用既有 Runtime Resolver。Admission 失敗時拒絕載入，live Player 與主要 UI 保持原狀；不自動修復、不刪除壞存檔。</x:v>
+      </x:c>
+      <x:c r="E12" t="str">
+        <x:v>career-save-admission.js；Save Admission tests；成年合法／非法 state matrix；atomic load／zero-live-mutation tests；legacy normalized save regression；loadGame integration；4.10 architecture document</x:v>
+      </x:c>
+      <x:c r="F12" t="str">
+        <x:v>合法 normalized adult save 才能替換 live Player；非法 careerExit／age／step／result-state contradiction 一律 rejected；rejected load 不修改 live Player、不呼叫 showCurrentEvent、不隱藏主要 UI、不刪 localStorage；合法 legacy save 經 normalize 後仍可 admission；SAVE_VERSION、Player Schema、Save Schema 均不變。</x:v>
+      </x:c>
+      <x:c r="G12" t="str">
+        <x:v>起始基線：23f3487
+Architecture Test Level C
+Adult Career Save Admission Integration</x:v>
+      </x:c>
       <x:c r="H12" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" t="str">
+        <x:v>4.11+</x:v>
+      </x:c>
+      <x:c r="B13"/>
+      <x:c r="C13" t="str">
+        <x:v>待 Architecture Sprint 4.10 結案後重新規劃</x:v>
+      </x:c>
+      <x:c r="D13"/>
+      <x:c r="E13"/>
+      <x:c r="F13"/>
+      <x:c r="G13"/>
+      <x:c r="H13" t="str">
         <x:v>待重新規劃</x:v>
       </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14"/>
+      <x:c r="B14"/>
+      <x:c r="C14"/>
+      <x:c r="D14"/>
+      <x:c r="E14"/>
+      <x:c r="F14"/>
+      <x:c r="G14"/>
+      <x:c r="H14"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15"/>
+      <x:c r="B15"/>
+      <x:c r="C15"/>
+      <x:c r="D15"/>
+      <x:c r="E15"/>
+      <x:c r="F15"/>
+      <x:c r="G15"/>
+      <x:c r="H15"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16"/>
+      <x:c r="B16"/>
+      <x:c r="C16"/>
+      <x:c r="D16"/>
+      <x:c r="E16"/>
+      <x:c r="F16"/>
+      <x:c r="G16"/>
+      <x:c r="H16"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17"/>
+      <x:c r="B17"/>
+      <x:c r="C17"/>
+      <x:c r="D17"/>
+      <x:c r="E17"/>
+      <x:c r="F17"/>
+      <x:c r="G17"/>
+      <x:c r="H17"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18"/>
+      <x:c r="B18"/>
+      <x:c r="C18"/>
+      <x:c r="D18"/>
+      <x:c r="E18"/>
+      <x:c r="F18"/>
+      <x:c r="G18"/>
+      <x:c r="H18"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19"/>
+      <x:c r="B19"/>
+      <x:c r="C19"/>
+      <x:c r="D19"/>
+      <x:c r="E19"/>
+      <x:c r="F19"/>
+      <x:c r="G19"/>
+      <x:c r="H19"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20"/>
+      <x:c r="B20"/>
+      <x:c r="C20"/>
+      <x:c r="D20"/>
+      <x:c r="E20"/>
+      <x:c r="F20"/>
+      <x:c r="G20"/>
+      <x:c r="H20"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21"/>
+      <x:c r="B21"/>
+      <x:c r="C21"/>
+      <x:c r="D21"/>
+      <x:c r="E21"/>
+      <x:c r="F21"/>
+      <x:c r="G21"/>
+      <x:c r="H21"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22"/>
+      <x:c r="B22"/>
+      <x:c r="C22"/>
+      <x:c r="D22"/>
+      <x:c r="E22"/>
+      <x:c r="F22"/>
+      <x:c r="G22"/>
+      <x:c r="H22"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23"/>
+      <x:c r="B23"/>
+      <x:c r="C23"/>
+      <x:c r="D23"/>
+      <x:c r="E23"/>
+      <x:c r="F23"/>
+      <x:c r="G23"/>
+      <x:c r="H23"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24"/>
+      <x:c r="B24"/>
+      <x:c r="C24"/>
+      <x:c r="D24"/>
+      <x:c r="E24"/>
+      <x:c r="F24"/>
+      <x:c r="G24"/>
+      <x:c r="H24"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25"/>
+      <x:c r="B25"/>
+      <x:c r="C25"/>
+      <x:c r="D25"/>
+      <x:c r="E25"/>
+      <x:c r="F25"/>
+      <x:c r="G25"/>
+      <x:c r="H25"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26"/>
+      <x:c r="B26"/>
+      <x:c r="C26"/>
+      <x:c r="D26"/>
+      <x:c r="E26"/>
+      <x:c r="F26"/>
+      <x:c r="G26"/>
+      <x:c r="H26"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27"/>
+      <x:c r="B27"/>
+      <x:c r="C27"/>
+      <x:c r="D27"/>
+      <x:c r="E27"/>
+      <x:c r="F27"/>
+      <x:c r="G27"/>
+      <x:c r="H27"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28"/>
+      <x:c r="B28"/>
+      <x:c r="C28"/>
+      <x:c r="D28"/>
+      <x:c r="E28"/>
+      <x:c r="F28"/>
+      <x:c r="G28"/>
+      <x:c r="H28"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29"/>
+      <x:c r="B29"/>
+      <x:c r="C29"/>
+      <x:c r="D29"/>
+      <x:c r="E29"/>
+      <x:c r="F29"/>
+      <x:c r="G29"/>
+      <x:c r="H29"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30"/>
+      <x:c r="B30"/>
+      <x:c r="C30"/>
+      <x:c r="D30"/>
+      <x:c r="E30"/>
+      <x:c r="F30"/>
+      <x:c r="G30"/>
+      <x:c r="H30"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31"/>
+      <x:c r="B31"/>
+      <x:c r="C31"/>
+      <x:c r="D31"/>
+      <x:c r="E31"/>
+      <x:c r="F31"/>
+      <x:c r="G31"/>
+      <x:c r="H31"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32"/>
+      <x:c r="B32"/>
+      <x:c r="C32"/>
+      <x:c r="D32"/>
+      <x:c r="E32"/>
+      <x:c r="F32"/>
+      <x:c r="G32"/>
+      <x:c r="H32"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33"/>
+      <x:c r="B33"/>
+      <x:c r="C33"/>
+      <x:c r="D33"/>
+      <x:c r="E33"/>
+      <x:c r="F33"/>
+      <x:c r="G33"/>
+      <x:c r="H33"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34"/>
+      <x:c r="B34"/>
+      <x:c r="C34"/>
+      <x:c r="D34"/>
+      <x:c r="E34"/>
+      <x:c r="F34"/>
+      <x:c r="G34"/>
+      <x:c r="H34"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35"/>
+      <x:c r="B35"/>
+      <x:c r="C35"/>
+      <x:c r="D35"/>
+      <x:c r="E35"/>
+      <x:c r="F35"/>
+      <x:c r="G35"/>
+      <x:c r="H35"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36"/>
+      <x:c r="B36"/>
+      <x:c r="C36"/>
+      <x:c r="D36"/>
+      <x:c r="E36"/>
+      <x:c r="F36"/>
+      <x:c r="G36"/>
+      <x:c r="H36"/>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37"/>
+      <x:c r="B37"/>
+      <x:c r="C37"/>
+      <x:c r="D37"/>
+      <x:c r="E37"/>
+      <x:c r="F37"/>
+      <x:c r="G37"/>
+      <x:c r="H37"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38"/>
+      <x:c r="B38"/>
+      <x:c r="C38"/>
+      <x:c r="D38"/>
+      <x:c r="E38"/>
+      <x:c r="F38"/>
+      <x:c r="G38"/>
+      <x:c r="H38"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39"/>
+      <x:c r="B39"/>
+      <x:c r="C39"/>
+      <x:c r="D39"/>
+      <x:c r="E39"/>
+      <x:c r="F39"/>
+      <x:c r="G39"/>
+      <x:c r="H39"/>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40"/>
+      <x:c r="B40"/>
+      <x:c r="C40"/>
+      <x:c r="D40"/>
+      <x:c r="E40"/>
+      <x:c r="F40"/>
+      <x:c r="G40"/>
+      <x:c r="H40"/>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41"/>
+      <x:c r="B41"/>
+      <x:c r="C41"/>
+      <x:c r="D41"/>
+      <x:c r="E41"/>
+      <x:c r="F41"/>
+      <x:c r="G41"/>
+      <x:c r="H41"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
feat: establish post-age-22 career rejoin contract
</commit_message>
<xml_diff>
--- a/棒球人生_三年設計排程_易讀版.xlsx
+++ b/棒球人生_三年設計排程_易讀版.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="R5b0218c1d7174dbf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R52c36708a5484917"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="Rc34b980a347e4a0f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R120101270eda430b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R5983230362ca427c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R30e6520caf3e43fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="Rdb7bd0c875294876"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R7ecf2474951a494b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="Refedbf6b84ad4429"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R7d9ba72a9fc44c4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="Red137465f2424e9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="Raa8bd5206f064311"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1356,7 +1356,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="13.800000190734863"/>
   <x:cols>
-    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="34" customWidth="1"/>
     <x:col min="3" max="8" width="13" customWidth="1"/>
     <x:col min="9" max="9" width="48" customWidth="1"/>
@@ -1609,22 +1609,21 @@
       <x:c r="G12" s="2"/>
       <x:c r="H12" s="2"/>
       <x:c r="I12" s="2" t="str">
-        <x:v>起始基線：23f3487
+        <x:v>起始基線：23f3487｜結案基線：543b845
 核心問題：一份 normalized 成年存檔在成為 live Player 前，誰負責證明它描述的是合法的 18–22 歲職涯位置？
-主要工作：建立 Adult Career Save Admission Boundary；以 CareerSpineContract 為主要狀態權威，並在生涯轉換期／發展期重用既有 Runtime Resolver；loadGame 先 normalize candidate，再 admission，只有 admitted 才能原子替換 live player。非法成年存檔拒絕載入且 live Player／主要 UI 不被污染，不自動修復、不自動刪除。
-測試級別：Architecture Test Level C／Adult Career Save Admission Integration
-排程：第一季追加 Sprint II</x:v>
+主要成果：建立 Adult Career Save Admission Boundary；loadGame 改為 parse → normalize candidate → admission → player assignment；只有 admitted 才能原子替換 live Player。非法成年存檔拒絕載入且 Player／主要 UI／Storage 不被污染；不自動修復、不自動刪除。
+測試級別：Architecture Test Level C／Adult Career Save Admission Integration</x:v>
       </x:c>
       <x:c r="J12" s="2" t="str">
         <x:v>完成</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
+    <x:row r="13" ht="100" customHeight="1">
       <x:c r="A13" s="30" t="str">
-        <x:v>4.11+</x:v>
+        <x:v>4.11</x:v>
       </x:c>
       <x:c r="B13" s="30" t="str">
-        <x:v>待 Architecture Sprint 4.10 結案後重新規劃</x:v>
+        <x:v>Architecture Sprint 4.11：Post-Age-22 Career Rejoin Readonly Contract</x:v>
       </x:c>
       <x:c r="C13" s="30"/>
       <x:c r="D13" s="30"/>
@@ -1632,16 +1631,25 @@
       <x:c r="F13" s="30"/>
       <x:c r="G13" s="30"/>
       <x:c r="H13" s="30"/>
-      <x:c r="I13" s="30"/>
+      <x:c r="I13" s="30" t="str">
+        <x:v>起始基線：543b845
+核心問題：22 歲職涯小結之後，哪些既有 route／future domain 可以形成可重新交會的候選職涯網路？
+鎖定拓樸：7 個 route/domain identity＝draft、college、amateur、rehab、professional、baseball-industry、player-competition；8 條 candidate edge 完全沿用 4.3 CareerSpineContract 既有 candidateTransitions。
+主要工作：新增唯讀 Post-Age-22 Career Rejoin Contract；從 CareerSpineContract.initialRoutes 與 candidateTransitions 導出節點與連線；標示 current endpoint、candidate-only、runtimePlayable=false；不得新增事件、chapter、Player／Save state，也不得接入 Runtime routing。
+測試級別：Architecture Test Level B／Readonly Future Career Topology Contract
+排程：第一季追加 Sprint III</x:v>
+      </x:c>
       <x:c r="J13" s="30" t="str">
-        <x:v>待重新規劃</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="36.75" customHeight="1">
-      <x:c r="A14" s="18" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="B14" s="5"/>
+      <x:c r="A14" s="18" t="str">
+        <x:v>4.12+</x:v>
+      </x:c>
+      <x:c r="B14" s="5" t="str">
+        <x:v>待 Architecture Sprint 4.11 結案後重新規劃</x:v>
+      </x:c>
       <x:c r="C14"/>
       <x:c r="D14"/>
       <x:c r="E14"/>
@@ -1649,15 +1657,15 @@
       <x:c r="G14"/>
       <x:c r="H14"/>
       <x:c r="I14"/>
-      <x:c r="J14"/>
+      <x:c r="J14" t="str">
+        <x:v>待重新規劃</x:v>
+      </x:c>
     </x:row>
     <x:row r="15" ht="36.75" customHeight="1">
       <x:c r="A15" s="19" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="B15" s="7" t="s">
-        <x:v>62</x:v>
-      </x:c>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B15" s="7"/>
       <x:c r="C15"/>
       <x:c r="D15"/>
       <x:c r="E15"/>
@@ -1669,10 +1677,10 @@
     </x:row>
     <x:row r="16" ht="36.75" customHeight="1">
       <x:c r="A16" s="19" t="s">
-        <x:v>63</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B16" s="7" t="s">
-        <x:v>64</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C16"/>
       <x:c r="D16"/>
@@ -1685,10 +1693,10 @@
     </x:row>
     <x:row r="17" ht="36.75" customHeight="1">
       <x:c r="A17" s="19" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B17" s="7" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C17"/>
       <x:c r="D17"/>
@@ -1701,10 +1709,10 @@
     </x:row>
     <x:row r="18" ht="36.75" customHeight="1">
       <x:c r="A18" s="20" t="s">
-        <x:v>67</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B18" s="10" t="s">
-        <x:v>68</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C18"/>
       <x:c r="D18"/>
@@ -1717,10 +1725,10 @@
     </x:row>
     <x:row r="19" ht="36.75" customHeight="1">
       <x:c r="A19" s="20" t="s">
-        <x:v>69</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B19" s="10" t="s">
-        <x:v>70</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C19"/>
       <x:c r="D19"/>
@@ -1733,10 +1741,10 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B20" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C20"/>
       <x:c r="D20"/>
@@ -1748,8 +1756,12 @@
       <x:c r="J20"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21"/>
-      <x:c r="B21"/>
+      <x:c r="A21" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B21" t="s">
+        <x:v>72</x:v>
+      </x:c>
       <x:c r="C21"/>
       <x:c r="D21"/>
       <x:c r="E21"/>
@@ -1998,6 +2010,30 @@
       <x:c r="H41"/>
       <x:c r="I41"/>
       <x:c r="J41"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42"/>
+      <x:c r="B42"/>
+      <x:c r="C42"/>
+      <x:c r="D42"/>
+      <x:c r="E42"/>
+      <x:c r="F42"/>
+      <x:c r="G42"/>
+      <x:c r="H42"/>
+      <x:c r="I42"/>
+      <x:c r="J42"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43"/>
+      <x:c r="B43"/>
+      <x:c r="C43"/>
+      <x:c r="D43"/>
+      <x:c r="E43"/>
+      <x:c r="F43"/>
+      <x:c r="G43"/>
+      <x:c r="H43"/>
+      <x:c r="I43"/>
+      <x:c r="J43"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2036,7 +2072,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="13.800000190734863"/>
   <x:cols>
-    <x:col min="1" max="1" width="9" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="13" customWidth="1"/>
     <x:col min="3" max="4" width="38" customWidth="1"/>
     <x:col min="5" max="5" width="42" customWidth="1"/>
@@ -2301,16 +2337,17 @@
         <x:v>一份 normalized 成年存檔在成為 live Player 前，誰負責證明它描述的是合法的 18–22 歲職涯位置？</x:v>
       </x:c>
       <x:c r="D12" t="str">
-        <x:v>建立 Adult Career Save Admission Boundary；在 normalizeSave() 之後、live player replacement 之前驗證成年 Career state。主要依據 CareerSpineContract；生涯轉換期與發展期再重用既有 Runtime Resolver。Admission 失敗時拒絕載入，live Player 與主要 UI 保持原狀；不自動修復、不刪除壞存檔。</x:v>
+        <x:v>建立 Adult Career Save Admission Boundary；在 normalizeSave() 之後、live player replacement 之前驗證成年 Career state。合法 candidate 才能原子替換 live Player；非法 candidate fail-closed。</x:v>
       </x:c>
       <x:c r="E12" t="str">
-        <x:v>career-save-admission.js；Save Admission tests；成年合法／非法 state matrix；atomic load／zero-live-mutation tests；legacy normalized save regression；loadGame integration；4.10 architecture document</x:v>
+        <x:v>career-save-admission.js；Save Admission tests；atomic load／zero-live-mutation tests；legacy normalized save regression；loadGame integration；4.10 architecture document</x:v>
       </x:c>
       <x:c r="F12" t="str">
-        <x:v>合法 normalized adult save 才能替換 live Player；非法 careerExit／age／step／result-state contradiction 一律 rejected；rejected load 不修改 live Player、不呼叫 showCurrentEvent、不隱藏主要 UI、不刪 localStorage；合法 legacy save 經 normalize 後仍可 admission；SAVE_VERSION、Player Schema、Save Schema 均不變。</x:v>
+        <x:v>合法 normalized adult save 才能替換 live Player；rejected load 不修改 Player identity/content、不呼叫 showCurrentEvent、不切換主要 UI、不改寫或刪除 Storage；SAVE_VERSION、Player／Save Schema 不變。</x:v>
       </x:c>
       <x:c r="G12" t="str">
         <x:v>起始基線：23f3487
+結案基線：543b845
 Architecture Test Level C
 Adult Career Save Admission Integration</x:v>
       </x:c>
@@ -2318,31 +2355,49 @@
         <x:v>完成</x:v>
       </x:c>
     </x:row>
-    <x:row r="13">
+    <x:row r="13" ht="60" customHeight="1">
       <x:c r="A13" t="str">
-        <x:v>4.11+</x:v>
-      </x:c>
-      <x:c r="B13"/>
+        <x:v>4.11</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>第一季追加 III</x:v>
+      </x:c>
       <x:c r="C13" t="str">
-        <x:v>待 Architecture Sprint 4.10 結案後重新規劃</x:v>
-      </x:c>
-      <x:c r="D13"/>
-      <x:c r="E13"/>
-      <x:c r="F13"/>
-      <x:c r="G13"/>
+        <x:v>22 歲職涯小結之後，哪些 route／future domain 可以形成可重新交會的候選職涯網路？</x:v>
+      </x:c>
+      <x:c r="D13" t="str">
+        <x:v>建立 Post-Age-22 Career Rejoin Readonly Contract。節點必須從既有 initialRoutes 與 candidateTransitions 導出；8 條 candidate edge 完全沿用 4.3 定義；正式區分 current endpoint、initial-route identity、future-only identity、candidate source/target。所有 22+ future topology 均明確 runtimePlayable=false，不接入 Gameplay。</x:v>
+      </x:c>
+      <x:c r="E13" t="str">
+        <x:v>career-rejoin-contract.js；Career Rejoin Contract tests；7-node／8-edge topology audit；candidate isolation tests；readonly／determinism tests；4.11 architecture document</x:v>
+      </x:c>
+      <x:c r="F13" t="str">
+        <x:v>7 個 route/domain identity 唯一且全部由既有 Contract 導出；8 條 candidate edge 與 4.3 candidateTransitions 一致；candidate 不得混入 actual edge、不得含 eventIds、不得被 Save Admission 視為現行合法 Runtime node；Player／Save／CareerSpineContract zero mutation，現有 Runtime routing 不變。</x:v>
+      </x:c>
+      <x:c r="G13" t="str">
+        <x:v>起始基線：543b845
+Architecture Test Level B
+Readonly Future Career Topology Contract</x:v>
+      </x:c>
       <x:c r="H13" t="str">
-        <x:v>待重新規劃</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14"/>
+      <x:c r="A14" t="str">
+        <x:v>4.12+</x:v>
+      </x:c>
       <x:c r="B14"/>
-      <x:c r="C14"/>
+      <x:c r="C14" t="str">
+        <x:v>待 Architecture Sprint 4.11 結案後重新規劃</x:v>
+      </x:c>
       <x:c r="D14"/>
       <x:c r="E14"/>
       <x:c r="F14"/>
       <x:c r="G14"/>
-      <x:c r="H14"/>
+      <x:c r="H14" t="str">
+        <x:v>待重新規劃</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15"/>
@@ -2613,6 +2668,26 @@
       <x:c r="F41"/>
       <x:c r="G41"/>
       <x:c r="H41"/>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42"/>
+      <x:c r="B42"/>
+      <x:c r="C42"/>
+      <x:c r="D42"/>
+      <x:c r="E42"/>
+      <x:c r="F42"/>
+      <x:c r="G42"/>
+      <x:c r="H42"/>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43"/>
+      <x:c r="B43"/>
+      <x:c r="C43"/>
+      <x:c r="D43"/>
+      <x:c r="E43"/>
+      <x:c r="F43"/>
+      <x:c r="G43"/>
+      <x:c r="H43"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
feat: establish age-22 career outcome classification boundary
</commit_message>
<xml_diff>
--- a/棒球人生_三年設計排程_易讀版.xlsx
+++ b/棒球人生_三年設計排程_易讀版.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="Rdb7bd0c875294876"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R7ecf2474951a494b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="Refedbf6b84ad4429"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R7d9ba72a9fc44c4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="Red137465f2424e9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="Raa8bd5206f064311"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="R61c1bfc5c32a4ad1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R71cdfe84c2c2494d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R998af974ca8c4a2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R7f068e61ea1746a3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R1bc8413d17dc4c25"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R1edbd372041f4579"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1356,7 +1356,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="13.800000190734863"/>
   <x:cols>
-    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="10" customWidth="1"/>
     <x:col min="2" max="2" width="34" customWidth="1"/>
     <x:col min="3" max="8" width="13" customWidth="1"/>
     <x:col min="9" max="9" width="48" customWidth="1"/>
@@ -1618,7 +1618,7 @@
         <x:v>完成</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="100" customHeight="1">
+    <x:row r="13">
       <x:c r="A13" s="30" t="str">
         <x:v>4.11</x:v>
       </x:c>
@@ -1632,12 +1632,9 @@
       <x:c r="G13" s="30"/>
       <x:c r="H13" s="30"/>
       <x:c r="I13" s="30" t="str">
-        <x:v>起始基線：543b845
-核心問題：22 歲職涯小結之後，哪些既有 route／future domain 可以形成可重新交會的候選職涯網路？
-鎖定拓樸：7 個 route/domain identity＝draft、college、amateur、rehab、professional、baseball-industry、player-competition；8 條 candidate edge 完全沿用 4.3 CareerSpineContract 既有 candidateTransitions。
-主要工作：新增唯讀 Post-Age-22 Career Rejoin Contract；從 CareerSpineContract.initialRoutes 與 candidateTransitions 導出節點與連線；標示 current endpoint、candidate-only、runtimePlayable=false；不得新增事件、chapter、Player／Save state，也不得接入 Runtime routing。
-測試級別：Architecture Test Level B／Readonly Future Career Topology Contract
-排程：第一季追加 Sprint III</x:v>
+        <x:v>起始基線：543b845｜結案基線：1782825
+核心成果：建立唯讀 22 歲後 Career Rejoin Future Topology；由既有 CareerSpineContract 的 initialRoutes 與 candidateTransitions 導出 7 identities／8 candidate edges；Future Contract 與目前 Runtime／Save Admission 完全隔離。
+測試級別：Architecture Test Level B／Readonly Future Career Topology Contract</x:v>
       </x:c>
       <x:c r="J13" s="30" t="str">
         <x:v>完成</x:v>
@@ -1645,10 +1642,10 @@
     </x:row>
     <x:row r="14" ht="36.75" customHeight="1">
       <x:c r="A14" s="18" t="str">
-        <x:v>4.12+</x:v>
+        <x:v>4.12</x:v>
       </x:c>
       <x:c r="B14" s="5" t="str">
-        <x:v>待 Architecture Sprint 4.11 結案後重新規劃</x:v>
+        <x:v>Architecture Sprint 4.12：Age-22 Career Outcome Classification Boundary</x:v>
       </x:c>
       <x:c r="C14"/>
       <x:c r="D14"/>
@@ -1656,16 +1653,26 @@
       <x:c r="F14"/>
       <x:c r="G14"/>
       <x:c r="H14"/>
-      <x:c r="I14"/>
+      <x:c r="I14" t="str">
+        <x:v>起始基線：1782825
+核心問題：22 歲既有八種結算結果如何取得穩定的 machine-readable outcome code 與 currentIdentity，而不解析中文文案或複製市場門檻？
+鎖定 outcome codes：professional-competitive、professional-roster-risk、college-draft-window、college-uncertain、amateur-professional-window、amateur-stable、rehab-player-reentry、rehab-second-career。
+currentIdentity：高卒兩個 careerExit → professional；大學棒球 → college；業餘／社會人棒球 → amateur；復健與生涯暫停 → rehab。
+主要工作：新增 readonly Age-22 Outcome Resolver，由 CareerSpineContract exact careerExit mapping 判定 route；evaluateDevelopmentYears 只計算既有 marketScore facts 並交給 Resolver；Resolver 單一擁有 12／11／10 與 injuryRisk≤4 分類門檻及八組既有結果文案。新增 persistent age22OutcomeCode；currentIdentity 不新增 Player 欄位，只由 Resolver 導出。Save v13→v14 做最小 deterministic migration。
+測試級別：Architecture Test Level B+／Readonly Age-22 Outcome Resolution Integration
+排程：第一季追加 Sprint IV</x:v>
+      </x:c>
       <x:c r="J14" t="str">
-        <x:v>待重新規劃</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="36.75" customHeight="1">
-      <x:c r="A15" s="19" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="B15" s="7"/>
+      <x:c r="A15" s="19" t="str">
+        <x:v>4.13+</x:v>
+      </x:c>
+      <x:c r="B15" s="7" t="str">
+        <x:v>待 Architecture Sprint 4.12 結案後重新規劃</x:v>
+      </x:c>
       <x:c r="C15"/>
       <x:c r="D15"/>
       <x:c r="E15"/>
@@ -1673,15 +1680,15 @@
       <x:c r="G15"/>
       <x:c r="H15"/>
       <x:c r="I15"/>
-      <x:c r="J15"/>
+      <x:c r="J15" t="str">
+        <x:v>待重新規劃</x:v>
+      </x:c>
     </x:row>
     <x:row r="16" ht="36.75" customHeight="1">
       <x:c r="A16" s="19" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="B16" s="7" t="s">
-        <x:v>62</x:v>
-      </x:c>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B16" s="7"/>
       <x:c r="C16"/>
       <x:c r="D16"/>
       <x:c r="E16"/>
@@ -1693,10 +1700,10 @@
     </x:row>
     <x:row r="17" ht="36.75" customHeight="1">
       <x:c r="A17" s="19" t="s">
-        <x:v>63</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B17" s="7" t="s">
-        <x:v>64</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C17"/>
       <x:c r="D17"/>
@@ -1709,10 +1716,10 @@
     </x:row>
     <x:row r="18" ht="36.75" customHeight="1">
       <x:c r="A18" s="20" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B18" s="10" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C18"/>
       <x:c r="D18"/>
@@ -1725,10 +1732,10 @@
     </x:row>
     <x:row r="19" ht="36.75" customHeight="1">
       <x:c r="A19" s="20" t="s">
-        <x:v>67</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B19" s="10" t="s">
-        <x:v>68</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C19"/>
       <x:c r="D19"/>
@@ -1741,10 +1748,10 @@
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="s">
-        <x:v>69</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B20" t="s">
-        <x:v>70</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C20"/>
       <x:c r="D20"/>
@@ -1757,10 +1764,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B21" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C21"/>
       <x:c r="D21"/>
@@ -1772,8 +1779,12 @@
       <x:c r="J21"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22"/>
-      <x:c r="B22"/>
+      <x:c r="A22" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B22" t="s">
+        <x:v>72</x:v>
+      </x:c>
       <x:c r="C22"/>
       <x:c r="D22"/>
       <x:c r="E22"/>
@@ -2034,6 +2045,30 @@
       <x:c r="H43"/>
       <x:c r="I43"/>
       <x:c r="J43"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44"/>
+      <x:c r="B44"/>
+      <x:c r="C44"/>
+      <x:c r="D44"/>
+      <x:c r="E44"/>
+      <x:c r="F44"/>
+      <x:c r="G44"/>
+      <x:c r="H44"/>
+      <x:c r="I44"/>
+      <x:c r="J44"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45"/>
+      <x:c r="B45"/>
+      <x:c r="C45"/>
+      <x:c r="D45"/>
+      <x:c r="E45"/>
+      <x:c r="F45"/>
+      <x:c r="G45"/>
+      <x:c r="H45"/>
+      <x:c r="I45"/>
+      <x:c r="J45"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2072,7 +2107,7 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="13.800000190734863"/>
   <x:cols>
-    <x:col min="1" max="1" width="11" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="9" customWidth="1"/>
     <x:col min="2" max="2" width="13" customWidth="1"/>
     <x:col min="3" max="4" width="38" customWidth="1"/>
     <x:col min="5" max="5" width="42" customWidth="1"/>
@@ -2355,7 +2390,7 @@
         <x:v>完成</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="60" customHeight="1">
+    <x:row r="13">
       <x:c r="A13" t="str">
         <x:v>4.11</x:v>
       </x:c>
@@ -2366,16 +2401,17 @@
         <x:v>22 歲職涯小結之後，哪些 route／future domain 可以形成可重新交會的候選職涯網路？</x:v>
       </x:c>
       <x:c r="D13" t="str">
-        <x:v>建立 Post-Age-22 Career Rejoin Readonly Contract。節點必須從既有 initialRoutes 與 candidateTransitions 導出；8 條 candidate edge 完全沿用 4.3 定義；正式區分 current endpoint、initial-route identity、future-only identity、candidate source/target。所有 22+ future topology 均明確 runtimePlayable=false，不接入 Gameplay。</x:v>
+        <x:v>建立 Post-Age-22 Career Rejoin Readonly Contract；由 initialRoutes 與 candidateTransitions 導出 7 identities／8 candidate edges；Future topology 不接 Runtime。</x:v>
       </x:c>
       <x:c r="E13" t="str">
-        <x:v>career-rejoin-contract.js；Career Rejoin Contract tests；7-node／8-edge topology audit；candidate isolation tests；readonly／determinism tests；4.11 architecture document</x:v>
+        <x:v>career-rejoin-contract.js；Career Rejoin Contract tests；7-node／8-edge topology audit；candidate isolation；readonly／determinism；4.11 architecture document</x:v>
       </x:c>
       <x:c r="F13" t="str">
-        <x:v>7 個 route/domain identity 唯一且全部由既有 Contract 導出；8 條 candidate edge 與 4.3 candidateTransitions 一致；candidate 不得混入 actual edge、不得含 eventIds、不得被 Save Admission 視為現行合法 Runtime node；Player／Save／CareerSpineContract zero mutation，現有 Runtime routing 不變。</x:v>
+        <x:v>Future topology 完全由既有 CareerSpineContract 導出；不 fabricated edge、不新增 event/chapter；Future identity 不成為 current Save state；Runtime／Save Admission zero impact。</x:v>
       </x:c>
       <x:c r="G13" t="str">
         <x:v>起始基線：543b845
+結案基線：1782825
 Architecture Test Level B
 Readonly Future Career Topology Contract</x:v>
       </x:c>
@@ -2385,29 +2421,47 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>4.12+</x:v>
-      </x:c>
-      <x:c r="B14"/>
+        <x:v>4.12</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>第一季追加 IV</x:v>
+      </x:c>
       <x:c r="C14" t="str">
-        <x:v>待 Architecture Sprint 4.11 結案後重新規劃</x:v>
-      </x:c>
-      <x:c r="D14"/>
-      <x:c r="E14"/>
-      <x:c r="F14"/>
-      <x:c r="G14"/>
+        <x:v>22 歲既有八種結算結果如何取得穩定的 outcome code 與 currentIdentity，而不讓文案或重複門檻成為未來路由真相？</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>建立 Age-22 Career Outcome Classification Boundary。Resolver 使用 CareerSpineContract exact careerExit mapping；evaluateDevelopmentYears 只提供既有 marketScore／injuryRisk facts；分類門檻與八組既有結果文案由 Resolver 單一擁有。新增 age22OutcomeCode；currentIdentity 為 derived result、不新增 Player 欄位。Save v13→v14 僅做最小 deterministic compatibility migration。</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>career-age22-outcome-resolver.js；Age-22 outcome tests；8-case classification matrix；currentIdentity mapping；evaluateDevelopmentYears integration；v13→v14 migration tests；Save Admission consistency regression；4.12 architecture document</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>8 個既有結果全部產生唯一穩定 age22OutcomeCode；高卒→professional、college→college、amateur→amateur、rehab→rehab；Runtime 不解析中文結果、不重複 12／11／10／injuryRisk≤4 門檻；v13 22歲存檔可安全升到 v14；v14 malformed/contradictory outcome code 不得成為可信 future-routing signal；4.11 Rejoin Contract 不修改、不做 Eligibility。</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>起始基線：1782825
+Architecture Test Level B+
+Readonly Age-22 Outcome Resolution Integration</x:v>
+      </x:c>
       <x:c r="H14" t="str">
-        <x:v>待重新規劃</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15"/>
+      <x:c r="A15" t="str">
+        <x:v>4.13+</x:v>
+      </x:c>
       <x:c r="B15"/>
-      <x:c r="C15"/>
+      <x:c r="C15" t="str">
+        <x:v>待 Architecture Sprint 4.12 結案後重新規劃</x:v>
+      </x:c>
       <x:c r="D15"/>
       <x:c r="E15"/>
       <x:c r="F15"/>
       <x:c r="G15"/>
-      <x:c r="H15"/>
+      <x:c r="H15" t="str">
+        <x:v>待重新規劃</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16"/>
@@ -2688,6 +2742,26 @@
       <x:c r="F43"/>
       <x:c r="G43"/>
       <x:c r="H43"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44"/>
+      <x:c r="B44"/>
+      <x:c r="C44"/>
+      <x:c r="D44"/>
+      <x:c r="E44"/>
+      <x:c r="F44"/>
+      <x:c r="G44"/>
+      <x:c r="H44"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45"/>
+      <x:c r="B45"/>
+      <x:c r="C45"/>
+      <x:c r="D45"/>
+      <x:c r="E45"/>
+      <x:c r="F45"/>
+      <x:c r="G45"/>
+      <x:c r="H45"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
feat: establish variable baseball situation prototype
</commit_message>
<xml_diff>
--- a/棒球人生_三年設計排程_易讀版.xlsx
+++ b/棒球人生_三年設計排程_易讀版.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="R61c1bfc5c32a4ad1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R71cdfe84c2c2494d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R998af974ca8c4a2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R7f068e61ea1746a3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R1bc8413d17dc4c25"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R1edbd372041f4579"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="R4c66600a29954c5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="Rc0a2b98099e84c53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R7c84e53bf0b64fe6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R7be8da7af8584aff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R7b118bd18b834864"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R66b187bb2543441f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -747,7 +747,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="37">
+  <x:cellXfs count="40">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -856,6 +856,15 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="11" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="2">
@@ -1660,51 +1669,63 @@
 currentIdentity：高卒兩個 careerExit → professional；大學棒球 → college；業餘／社會人棒球 → amateur；復健與生涯暫停 → rehab。
 主要工作：新增 readonly Age-22 Outcome Resolver，由 CareerSpineContract exact careerExit mapping 判定 route；evaluateDevelopmentYears 只計算既有 marketScore facts 並交給 Resolver；Resolver 單一擁有 12／11／10 與 injuryRisk≤4 分類門檻及八組既有結果文案。新增 persistent age22OutcomeCode；currentIdentity 不新增 Player 欄位，只由 Resolver 導出。Save v13→v14 做最小 deterministic migration。
 測試級別：Architecture Test Level B+／Readonly Age-22 Outcome Resolution Integration
-排程：第一季追加 Sprint IV</x:v>
+排程：第一季追加 Sprint IV
+結案基線：fe801fa</x:v>
       </x:c>
       <x:c r="J14" t="str">
         <x:v>完成</x:v>
       </x:c>
     </x:row>
-    <x:row r="15" ht="36.75" customHeight="1">
-      <x:c r="A15" s="19" t="str">
+    <x:row r="15" ht="95" customHeight="1">
+      <x:c r="A15" s="37" t="str">
+        <x:v>5.1</x:v>
+      </x:c>
+      <x:c r="B15" s="38" t="str">
+        <x:v>Gameplay Sprint 5.1：Variable Baseball Situation Core Loop Prototype</x:v>
+      </x:c>
+      <x:c r="C15" s="39"/>
+      <x:c r="D15" s="39"/>
+      <x:c r="E15" s="39"/>
+      <x:c r="F15" s="39"/>
+      <x:c r="G15" s="39"/>
+      <x:c r="H15" s="39"/>
+      <x:c r="I15" s="39" t="str">
+        <x:v>起始基線：fe801fa
+階段：Gameplay Validation
+承接基礎：Career Architecture Foundation v1（Architecture 4.3～4.12，暫時完成／封存為 Gameplay Validation 前安全基礎）
+核心工作：Offensive Prototype A；Defensive Prototype B；Isolated Sandbox；Deterministic Resolver；Debug Trace；Zero Production Integration
+測試級別：Gameplay Test Level B+／Isolated Variable Situation Prototype</x:v>
+      </x:c>
+      <x:c r="J15" s="39" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="42" customHeight="1">
+      <x:c r="A16" s="37" t="str">
         <x:v>4.13+</x:v>
       </x:c>
-      <x:c r="B15" s="7" t="str">
-        <x:v>待 Architecture Sprint 4.12 結案後重新規劃</x:v>
-      </x:c>
-      <x:c r="C15"/>
-      <x:c r="D15"/>
-      <x:c r="E15"/>
-      <x:c r="F15"/>
-      <x:c r="G15"/>
-      <x:c r="H15"/>
-      <x:c r="I15"/>
-      <x:c r="J15" t="str">
-        <x:v>待重新規劃</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="36.75" customHeight="1">
-      <x:c r="A16" s="19" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="B16" s="7"/>
-      <x:c r="C16"/>
-      <x:c r="D16"/>
-      <x:c r="E16"/>
-      <x:c r="F16"/>
-      <x:c r="G16"/>
-      <x:c r="H16"/>
-      <x:c r="I16"/>
-      <x:c r="J16"/>
+      <x:c r="B16" s="38" t="str">
+        <x:v>Post-Age-22 Architecture Expansion</x:v>
+      </x:c>
+      <x:c r="C16" s="39"/>
+      <x:c r="D16" s="39"/>
+      <x:c r="E16" s="39"/>
+      <x:c r="F16" s="39"/>
+      <x:c r="G16" s="39"/>
+      <x:c r="H16" s="39"/>
+      <x:c r="I16" s="39" t="str">
+        <x:v>Deferred pending Gameplay Validation
+目前不排 Eligibility 施工日期。</x:v>
+      </x:c>
+      <x:c r="J16" s="39" t="str">
+        <x:v>延後</x:v>
+      </x:c>
     </x:row>
     <x:row r="17" ht="36.75" customHeight="1">
       <x:c r="A17" s="19" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="B17" s="7" t="s">
-        <x:v>62</x:v>
-      </x:c>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B17" s="7"/>
       <x:c r="C17"/>
       <x:c r="D17"/>
       <x:c r="E17"/>
@@ -1716,10 +1737,10 @@
     </x:row>
     <x:row r="18" ht="36.75" customHeight="1">
       <x:c r="A18" s="20" t="s">
-        <x:v>63</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B18" s="10" t="s">
-        <x:v>64</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C18"/>
       <x:c r="D18"/>
@@ -1732,10 +1753,10 @@
     </x:row>
     <x:row r="19" ht="36.75" customHeight="1">
       <x:c r="A19" s="20" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B19" s="10" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C19"/>
       <x:c r="D19"/>
@@ -1746,12 +1767,12 @@
       <x:c r="I19"/>
       <x:c r="J19"/>
     </x:row>
-    <x:row r="20">
+    <x:row r="20" ht="36.75" customHeight="1">
       <x:c r="A20" t="s">
-        <x:v>67</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B20" t="s">
-        <x:v>68</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C20"/>
       <x:c r="D20"/>
@@ -1764,10 +1785,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="s">
-        <x:v>69</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B21" t="s">
-        <x:v>70</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C21"/>
       <x:c r="D21"/>
@@ -1780,10 +1801,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B22" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C22"/>
       <x:c r="D22"/>
@@ -1795,8 +1816,12 @@
       <x:c r="J22"/>
     </x:row>
     <x:row r="23">
-      <x:c r="A23"/>
-      <x:c r="B23"/>
+      <x:c r="A23" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B23" t="s">
+        <x:v>72</x:v>
+      </x:c>
       <x:c r="C23"/>
       <x:c r="D23"/>
       <x:c r="E23"/>
@@ -2069,6 +2094,18 @@
       <x:c r="H45"/>
       <x:c r="I45"/>
       <x:c r="J45"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46"/>
+      <x:c r="B46"/>
+      <x:c r="C46"/>
+      <x:c r="D46"/>
+      <x:c r="E46"/>
+      <x:c r="F46"/>
+      <x:c r="G46"/>
+      <x:c r="H46"/>
+      <x:c r="I46"/>
+      <x:c r="J46"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2441,37 +2478,59 @@
       <x:c r="G14" t="str">
         <x:v>起始基線：1782825
 Architecture Test Level B+
-Readonly Age-22 Outcome Resolution Integration</x:v>
+Readonly Age-22 Outcome Resolution Integration
+結案基線：fe801fa</x:v>
       </x:c>
       <x:c r="H14" t="str">
         <x:v>完成</x:v>
       </x:c>
     </x:row>
-    <x:row r="15">
-      <x:c r="A15" t="str">
+    <x:row r="15" ht="132" customHeight="1">
+      <x:c r="A15" s="39" t="str">
+        <x:v>5.1</x:v>
+      </x:c>
+      <x:c r="B15" s="39" t="str">
+        <x:v>Gameplay Validation I</x:v>
+      </x:c>
+      <x:c r="C15" s="39" t="str">
+        <x:v>固定棒球規則下，同一組選項能否因局勢、能力、身體與對手條件不同而改變價值，並產生可解釋但不固定的結果？</x:v>
+      </x:c>
+      <x:c r="D15" s="39" t="str">
+        <x:v>建立完全隔離的攻擊打席與內野守備兩階段 Prototype；Decision Quality 與 Execution 分離；所有 RNG 由 caller 注入；輸出 machine-readable state delta；正式 Runtime zero integration。</x:v>
+      </x:c>
+      <x:c r="E15" s="39" t="str">
+        <x:v>baseball-offense-prototype.js；baseball-defense-prototype.js；prototype utils；isolated sandbox page／CSS／controller；Offense／Defense／Isolation tests；5.1 design document</x:v>
+      </x:c>
+      <x:c r="F15" s="39" t="str">
+        <x:v>攻擊與守備 core deterministic、deep frozen、zero mutation；12-case offensive／defensive matrices 通過；好決策可壞結果、差決策可好執行；Run 10 有受模型約束的波動；正式 Player／Save／Story／Storage 不受影響。</x:v>
+      </x:c>
+      <x:c r="G15" s="39" t="str">
+        <x:v>起始基線：fe801fa
+Gameplay Test Level B+
+Isolated Variable Situation Prototype
+Career Architecture Foundation v1：Architecture 4.3～4.12 暫時完成／封存</x:v>
+      </x:c>
+      <x:c r="H15" s="39" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="48" customHeight="1">
+      <x:c r="A16" s="39" t="str">
         <x:v>4.13+</x:v>
       </x:c>
-      <x:c r="B15"/>
-      <x:c r="C15" t="str">
-        <x:v>待 Architecture Sprint 4.12 結案後重新規劃</x:v>
-      </x:c>
-      <x:c r="D15"/>
-      <x:c r="E15"/>
-      <x:c r="F15"/>
-      <x:c r="G15"/>
-      <x:c r="H15" t="str">
-        <x:v>待重新規劃</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16"/>
-      <x:c r="B16"/>
-      <x:c r="C16"/>
-      <x:c r="D16"/>
-      <x:c r="E16"/>
-      <x:c r="F16"/>
-      <x:c r="G16"/>
-      <x:c r="H16"/>
+      <x:c r="B16" s="39"/>
+      <x:c r="C16" s="39" t="str">
+        <x:v>Post-Age-22 Architecture Expansion／Deferred pending Gameplay Validation</x:v>
+      </x:c>
+      <x:c r="D16" s="39"/>
+      <x:c r="E16" s="39"/>
+      <x:c r="F16" s="39" t="str">
+        <x:v>不排 Eligibility 施工日期；不在本 Sprint 規劃 Gameplay Sprint 5.2。</x:v>
+      </x:c>
+      <x:c r="G16" s="39"/>
+      <x:c r="H16" s="39" t="str">
+        <x:v>延後</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17"/>

</xml_diff>

<commit_message>
feat: integrate first variable baseball gameplay event
</commit_message>
<xml_diff>
--- a/棒球人生_三年設計排程_易讀版.xlsx
+++ b/棒球人生_三年設計排程_易讀版.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="R4c66600a29954c5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="Rc0a2b98099e84c53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R7c84e53bf0b64fe6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R7be8da7af8584aff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R7b118bd18b834864"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R66b187bb2543441f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="Re5fb86762979460d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R6442cc5797e54fb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R61ac7da0d7694d45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R8bd5c0bfefd24e2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="Rf375917e3c384ee2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R0631ed42d25a4b72"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1694,18 +1694,19 @@
 階段：Gameplay Validation
 承接基礎：Career Architecture Foundation v1（Architecture 4.3～4.12，暫時完成／封存為 Gameplay Validation 前安全基礎）
 核心工作：Offensive Prototype A；Defensive Prototype B；Isolated Sandbox；Deterministic Resolver；Debug Trace；Zero Production Integration
-測試級別：Gameplay Test Level B+／Isolated Variable Situation Prototype</x:v>
+測試級別：Gameplay Test Level B+／Isolated Variable Situation Prototype
+結案基線：8e58b51</x:v>
       </x:c>
       <x:c r="J15" s="39" t="str">
         <x:v>完成</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="42" customHeight="1">
+    <x:row r="16" ht="116" customHeight="1">
       <x:c r="A16" s="37" t="str">
-        <x:v>4.13+</x:v>
+        <x:v>5.2</x:v>
       </x:c>
       <x:c r="B16" s="38" t="str">
-        <x:v>Post-Age-22 Architecture Expansion</x:v>
+        <x:v>Gameplay Sprint 5.2：Baseball Gameplay Integration Pilot</x:v>
       </x:c>
       <x:c r="C16" s="39"/>
       <x:c r="D16" s="39"/>
@@ -1714,34 +1715,41 @@
       <x:c r="G16" s="39"/>
       <x:c r="H16" s="39"/>
       <x:c r="I16" s="39" t="str">
-        <x:v>Deferred pending Gameplay Validation
-目前不排 Eligibility 施工日期。</x:v>
+        <x:v>起始基線：8e58b51
+階段：Gameplay Validation
+核心工作：First Production Gameplay Integration；youth_match_grounder live pilot；high_school_year_two_spring_game readiness-only
+測試級別：Gameplay Test Level C／First Production Gameplay Mutation Integration</x:v>
       </x:c>
       <x:c r="J16" s="39" t="str">
-        <x:v>延後</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="36.75" customHeight="1">
-      <x:c r="A17" s="19" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="B17" s="7"/>
+      <x:c r="A17" s="19" t="str">
+        <x:v>4.13+</x:v>
+      </x:c>
+      <x:c r="B17" s="7" t="str">
+        <x:v>Post-Age-22 Architecture Expansion</x:v>
+      </x:c>
       <x:c r="C17"/>
       <x:c r="D17"/>
       <x:c r="E17"/>
       <x:c r="F17"/>
       <x:c r="G17"/>
       <x:c r="H17"/>
-      <x:c r="I17"/>
-      <x:c r="J17"/>
+      <x:c r="I17" t="str">
+        <x:v>Deferred pending Gameplay Validation
+目前不排 Eligibility 施工日期；後續 Gameplay Sprint 日期未規劃。</x:v>
+      </x:c>
+      <x:c r="J17" t="str">
+        <x:v>延後</x:v>
+      </x:c>
     </x:row>
     <x:row r="18" ht="36.75" customHeight="1">
       <x:c r="A18" s="20" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="B18" s="10" t="s">
-        <x:v>62</x:v>
-      </x:c>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B18" s="10"/>
       <x:c r="C18"/>
       <x:c r="D18"/>
       <x:c r="E18"/>
@@ -1753,10 +1761,10 @@
     </x:row>
     <x:row r="19" ht="36.75" customHeight="1">
       <x:c r="A19" s="20" t="s">
-        <x:v>63</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B19" s="10" t="s">
-        <x:v>64</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C19"/>
       <x:c r="D19"/>
@@ -1769,10 +1777,10 @@
     </x:row>
     <x:row r="20" ht="36.75" customHeight="1">
       <x:c r="A20" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B20" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C20"/>
       <x:c r="D20"/>
@@ -1785,10 +1793,10 @@
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="s">
-        <x:v>67</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B21" t="s">
-        <x:v>68</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C21"/>
       <x:c r="D21"/>
@@ -1801,10 +1809,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="s">
-        <x:v>69</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B22" t="s">
-        <x:v>70</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C22"/>
       <x:c r="D22"/>
@@ -1817,10 +1825,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B23" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C23"/>
       <x:c r="D23"/>
@@ -1832,8 +1840,12 @@
       <x:c r="J23"/>
     </x:row>
     <x:row r="24">
-      <x:c r="A24"/>
-      <x:c r="B24"/>
+      <x:c r="A24" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B24" t="s">
+        <x:v>72</x:v>
+      </x:c>
       <x:c r="C24"/>
       <x:c r="D24"/>
       <x:c r="E24"/>
@@ -2106,6 +2118,18 @@
       <x:c r="H46"/>
       <x:c r="I46"/>
       <x:c r="J46"/>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47"/>
+      <x:c r="B47"/>
+      <x:c r="C47"/>
+      <x:c r="D47"/>
+      <x:c r="E47"/>
+      <x:c r="F47"/>
+      <x:c r="G47"/>
+      <x:c r="H47"/>
+      <x:c r="I47"/>
+      <x:c r="J47"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2508,39 +2532,58 @@
         <x:v>起始基線：fe801fa
 Gameplay Test Level B+
 Isolated Variable Situation Prototype
-Career Architecture Foundation v1：Architecture 4.3～4.12 暫時完成／封存</x:v>
+Career Architecture Foundation v1：Architecture 4.3～4.12 暫時完成／封存
+結案基線：8e58b51</x:v>
       </x:c>
       <x:c r="H15" s="39" t="str">
         <x:v>完成</x:v>
       </x:c>
     </x:row>
-    <x:row r="16" ht="48" customHeight="1">
+    <x:row r="16" ht="132" customHeight="1">
       <x:c r="A16" s="39" t="str">
+        <x:v>5.2</x:v>
+      </x:c>
+      <x:c r="B16" s="39" t="str">
+        <x:v>Gameplay Validation II</x:v>
+      </x:c>
+      <x:c r="C16" s="39" t="str">
+        <x:v>5.1 deterministic Gameplay Core 能否安全接入一個正式 Story Event，同時保持 progression、Outcome、Player state 與 Save flow 正常？</x:v>
+      </x:c>
+      <x:c r="D16" s="39" t="str">
+        <x:v>建立 BaseballGameplayIntegration 單一 adapter；將 youth_match_grounder 改為接球與傳球兩階段；Core 結果由 script.js exactly once 寫入正式 matchState 與球季結果；高中春季打擊只做 Base State readiness 判定。</x:v>
+      </x:c>
+      <x:c r="E16" s="39" t="str">
+        <x:v>baseball-gameplay-integration.js；Integration tests；正式兩階段 Grounder UI；result-specific continuity flags；Save pending guard；5.2 architecture document</x:v>
+      </x:c>
+      <x:c r="F16" s="39" t="str">
+        <x:v>youth_match_grounder 真正使用 Defensive Core；Choice 不固定決定出局、失誤或雙殺；Stage A 影響 Stage B；Outcome 等待 Continue；其他少棒守位與高中打擊 Gameplay 不變。</x:v>
+      </x:c>
+      <x:c r="G16" s="39" t="str">
+        <x:v>起始基線：8e58b51
+Gameplay Test Level C
+First Production Gameplay Mutation Integration</x:v>
+      </x:c>
+      <x:c r="H16" s="39" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" t="str">
         <x:v>4.13+</x:v>
       </x:c>
-      <x:c r="B16" s="39"/>
-      <x:c r="C16" s="39" t="str">
+      <x:c r="B17"/>
+      <x:c r="C17" t="str">
         <x:v>Post-Age-22 Architecture Expansion／Deferred pending Gameplay Validation</x:v>
       </x:c>
-      <x:c r="D16" s="39"/>
-      <x:c r="E16" s="39"/>
-      <x:c r="F16" s="39" t="str">
-        <x:v>不排 Eligibility 施工日期；不在本 Sprint 規劃 Gameplay Sprint 5.2。</x:v>
-      </x:c>
-      <x:c r="G16" s="39"/>
-      <x:c r="H16" s="39" t="str">
-        <x:v>延後</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17"/>
-      <x:c r="B17"/>
-      <x:c r="C17"/>
       <x:c r="D17"/>
       <x:c r="E17"/>
-      <x:c r="F17"/>
+      <x:c r="F17" t="str">
+        <x:v>不排 Eligibility 施工日期；後續 Gameplay Sprint 日期未規劃。</x:v>
+      </x:c>
       <x:c r="G17"/>
-      <x:c r="H17"/>
+      <x:c r="H17" t="str">
+        <x:v>延後</x:v>
+      </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18"/>
@@ -2821,6 +2864,16 @@
       <x:c r="F45"/>
       <x:c r="G45"/>
       <x:c r="H45"/>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46"/>
+      <x:c r="B46"/>
+      <x:c r="C46"/>
+      <x:c r="D46"/>
+      <x:c r="E46"/>
+      <x:c r="F46"/>
+      <x:c r="G46"/>
+      <x:c r="H46"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
feat: expand offensive gameplay base states
</commit_message>
<xml_diff>
--- a/棒球人生_三年設計排程_易讀版.xlsx
+++ b/棒球人生_三年設計排程_易讀版.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="Re5fb86762979460d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R6442cc5797e54fb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R61ac7da0d7694d45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R8bd5c0bfefd24e2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="Rf375917e3c384ee2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R0631ed42d25a4b72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="Rb817ad5c03fd41cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R288c60a355294d41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R3fcf128245bf4828"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R15159e9f9c6846dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R1956c5d8f16c44be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="Red3494e4845d4d44"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1718,18 +1718,19 @@
         <x:v>起始基線：8e58b51
 階段：Gameplay Validation
 核心工作：First Production Gameplay Integration；youth_match_grounder live pilot；high_school_year_two_spring_game readiness-only
-測試級別：Gameplay Test Level C／First Production Gameplay Mutation Integration</x:v>
+測試級別：Gameplay Test Level C／First Production Gameplay Mutation Integration
+結案基線：028cffb</x:v>
       </x:c>
       <x:c r="J16" s="39" t="str">
         <x:v>完成</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="36.75" customHeight="1">
+    <x:row r="17" ht="92" customHeight="1">
       <x:c r="A17" s="19" t="str">
-        <x:v>4.13+</x:v>
+        <x:v>5.3</x:v>
       </x:c>
       <x:c r="B17" s="7" t="str">
-        <x:v>Post-Age-22 Architecture Expansion</x:v>
+        <x:v>Gameplay Sprint 5.3：Offensive Base-State Expansion</x:v>
       </x:c>
       <x:c r="C17"/>
       <x:c r="D17"/>
@@ -1738,34 +1739,41 @@
       <x:c r="G17"/>
       <x:c r="H17"/>
       <x:c r="I17" t="str">
-        <x:v>Deferred pending Gameplay Validation
-目前不排 Eligibility 施工日期；後續 Gameplay Sprint 日期未規劃。</x:v>
+        <x:v>起始基線：028cffb
+階段：Gameplay Validation III
+核心工作：one-out-runner-on-first＋one-out-runner-on-second；Base-State-aware Decision／Result／State Delta；high_school_year_two_spring_game readiness-only compatible
+測試級別：Gameplay Test Level B+／Offensive Base-State Model Expansion</x:v>
       </x:c>
       <x:c r="J17" t="str">
-        <x:v>延後</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="36.75" customHeight="1">
-      <x:c r="A18" s="20" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="B18" s="10"/>
+      <x:c r="A18" s="20" t="str">
+        <x:v>4.13+</x:v>
+      </x:c>
+      <x:c r="B18" s="10" t="str">
+        <x:v>Post-Age-22 Architecture Expansion</x:v>
+      </x:c>
       <x:c r="C18"/>
       <x:c r="D18"/>
       <x:c r="E18"/>
       <x:c r="F18"/>
       <x:c r="G18"/>
       <x:c r="H18"/>
-      <x:c r="I18"/>
-      <x:c r="J18"/>
+      <x:c r="I18" t="str">
+        <x:v>Deferred pending Gameplay Validation
+目前不排 Eligibility 施工日期；後續 Gameplay Sprint 日期未規劃。</x:v>
+      </x:c>
+      <x:c r="J18" t="str">
+        <x:v>延後</x:v>
+      </x:c>
     </x:row>
     <x:row r="19" ht="36.75" customHeight="1">
       <x:c r="A19" s="20" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="B19" s="10" t="s">
-        <x:v>62</x:v>
-      </x:c>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B19" s="10"/>
       <x:c r="C19"/>
       <x:c r="D19"/>
       <x:c r="E19"/>
@@ -1777,10 +1785,10 @@
     </x:row>
     <x:row r="20" ht="36.75" customHeight="1">
       <x:c r="A20" t="s">
-        <x:v>63</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B20" t="s">
-        <x:v>64</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C20"/>
       <x:c r="D20"/>
@@ -1791,12 +1799,12 @@
       <x:c r="I20"/>
       <x:c r="J20"/>
     </x:row>
-    <x:row r="21">
+    <x:row r="21" ht="36.75" customHeight="1">
       <x:c r="A21" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B21" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C21"/>
       <x:c r="D21"/>
@@ -1809,10 +1817,10 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="s">
-        <x:v>67</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B22" t="s">
-        <x:v>68</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C22"/>
       <x:c r="D22"/>
@@ -1825,10 +1833,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="s">
-        <x:v>69</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B23" t="s">
-        <x:v>70</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C23"/>
       <x:c r="D23"/>
@@ -1841,10 +1849,10 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B24" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C24"/>
       <x:c r="D24"/>
@@ -1856,8 +1864,12 @@
       <x:c r="J24"/>
     </x:row>
     <x:row r="25">
-      <x:c r="A25"/>
-      <x:c r="B25"/>
+      <x:c r="A25" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B25" t="s">
+        <x:v>72</x:v>
+      </x:c>
       <x:c r="C25"/>
       <x:c r="D25"/>
       <x:c r="E25"/>
@@ -2561,39 +2573,58 @@
       <x:c r="G16" s="39" t="str">
         <x:v>起始基線：8e58b51
 Gameplay Test Level C
-First Production Gameplay Mutation Integration</x:v>
+First Production Gameplay Mutation Integration
+結案基線：028cffb</x:v>
       </x:c>
       <x:c r="H16" s="39" t="str">
         <x:v>完成</x:v>
       </x:c>
     </x:row>
-    <x:row r="17">
+    <x:row r="17" ht="116" customHeight="1">
       <x:c r="A17" t="str">
+        <x:v>5.3</x:v>
+      </x:c>
+      <x:c r="B17" t="str">
+        <x:v>Gameplay Validation III</x:v>
+      </x:c>
+      <x:c r="C17" t="str">
+        <x:v>Offensive Core 能否在不接入正式 Runtime 的前提下，同時支援一出局一壘與一出局二壘，並讓壘況具體改變決策、結果與跑者推進？</x:v>
+      </x:c>
+      <x:c r="D17" t="str">
+        <x:v>擴充精確 Base State API；建立 Base-State-aware Decision／Result／State Delta；保留一壘既有機率；新增二壘滾地、安打、觸擊與跑者推進模型；高中春季打擊僅由不相容改為 readiness-only compatible。</x:v>
+      </x:c>
+      <x:c r="E17" t="str">
+        <x:v>baseball-offense-prototype.js；baseball-gameplay-integration.js；Sandbox Base State selector；Offensive Base State tests；5.3 design document</x:v>
+      </x:c>
+      <x:c r="F17" t="str">
+        <x:v>支援 one-out-runner-on-first 與 one-out-runner-on-second；未知 Base State fail closed；runnersAfter 成為通用壘況真相；一壘回歸不變；二壘不產生一般雙殺或野選；正式 Player／Save／Story／Runtime mutation 維持不變。</x:v>
+      </x:c>
+      <x:c r="G17" t="str">
+        <x:v>起始基線：028cffb
+Gameplay Test Level B+
+Offensive Base-State Model Expansion</x:v>
+      </x:c>
+      <x:c r="H17" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" t="str">
         <x:v>4.13+</x:v>
       </x:c>
-      <x:c r="B17"/>
-      <x:c r="C17" t="str">
+      <x:c r="B18"/>
+      <x:c r="C18" t="str">
         <x:v>Post-Age-22 Architecture Expansion／Deferred pending Gameplay Validation</x:v>
       </x:c>
-      <x:c r="D17"/>
-      <x:c r="E17"/>
-      <x:c r="F17" t="str">
-        <x:v>不排 Eligibility 施工日期；後續 Gameplay Sprint 日期未規劃。</x:v>
-      </x:c>
-      <x:c r="G17"/>
-      <x:c r="H17" t="str">
-        <x:v>延後</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18"/>
-      <x:c r="B18"/>
-      <x:c r="C18"/>
       <x:c r="D18"/>
       <x:c r="E18"/>
-      <x:c r="F18"/>
+      <x:c r="F18" t="str">
+        <x:v>不排 Eligibility 施工日期；後續 Gameplay Sprint 日期未規劃。</x:v>
+      </x:c>
       <x:c r="G18"/>
-      <x:c r="H18"/>
+      <x:c r="H18" t="str">
+        <x:v>延後</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19"/>

</xml_diff>

<commit_message>
feat: integrate first offensive baseball gameplay event
</commit_message>
<xml_diff>
--- a/棒球人生_三年設計排程_易讀版.xlsx
+++ b/棒球人生_三年設計排程_易讀版.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="Rb817ad5c03fd41cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R288c60a355294d41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R3fcf128245bf4828"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R15159e9f9c6846dc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R1956c5d8f16c44be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="Red3494e4845d4d44"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="R6ac572880fa04d93"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R87b4ad8228004c2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R46ca32390d8f4a52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R3d4b07bbbaec4b1c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R19bc198f2bb04ecd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="Ra95f9b092aa4476d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1739,21 +1739,21 @@
       <x:c r="G17"/>
       <x:c r="H17"/>
       <x:c r="I17" t="str">
-        <x:v>起始基線：028cffb
+        <x:v>起始基線：028cffb｜結案基線：3b50316
 階段：Gameplay Validation III
-核心工作：one-out-runner-on-first＋one-out-runner-on-second；Base-State-aware Decision／Result／State Delta；high_school_year_two_spring_game readiness-only compatible
+核心工作：one-out-runner-on-first＋one-out-runner-on-second；Base-State-aware Decision／Result／State Delta；高中春季打擊維持 readiness-only。
 測試級別：Gameplay Test Level B+／Offensive Base-State Model Expansion</x:v>
       </x:c>
       <x:c r="J17" t="str">
         <x:v>完成</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="36.75" customHeight="1">
+    <x:row r="18" ht="92" customHeight="1">
       <x:c r="A18" s="20" t="str">
-        <x:v>4.13+</x:v>
+        <x:v>5.4</x:v>
       </x:c>
       <x:c r="B18" s="10" t="str">
-        <x:v>Post-Age-22 Architecture Expansion</x:v>
+        <x:v>Gameplay Sprint 5.4：First Offensive Production Integration</x:v>
       </x:c>
       <x:c r="C18"/>
       <x:c r="D18"/>
@@ -1762,34 +1762,41 @@
       <x:c r="G18"/>
       <x:c r="H18"/>
       <x:c r="I18" t="str">
-        <x:v>Deferred pending Gameplay Validation
-目前不排 Eligibility 施工日期；後續 Gameplay Sprint 日期未規劃。</x:v>
+        <x:v>起始基線：3b50316
+階段：Gameplay Validation IV
+核心工作：high_school_year_two_spring_game live integration；one-out-runner-on-second；Offensive Core → Player Match State。
+測試級別：Gameplay Test Level C／First Production Offensive Mutation Integration</x:v>
       </x:c>
       <x:c r="J18" t="str">
-        <x:v>延後</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="36.75" customHeight="1">
-      <x:c r="A19" s="20" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="B19" s="10"/>
+      <x:c r="A19" s="20" t="str">
+        <x:v>4.13+</x:v>
+      </x:c>
+      <x:c r="B19" s="10" t="str">
+        <x:v>Post-Age-22 Architecture Expansion</x:v>
+      </x:c>
       <x:c r="C19"/>
       <x:c r="D19"/>
       <x:c r="E19"/>
       <x:c r="F19"/>
       <x:c r="G19"/>
       <x:c r="H19"/>
-      <x:c r="I19"/>
-      <x:c r="J19"/>
+      <x:c r="I19" t="str">
+        <x:v>Deferred pending Gameplay Validation
+目前不排 Eligibility 施工日期；後續 Gameplay Sprint 日期未規劃。</x:v>
+      </x:c>
+      <x:c r="J19" t="str">
+        <x:v>延後</x:v>
+      </x:c>
     </x:row>
     <x:row r="20" ht="36.75" customHeight="1">
       <x:c r="A20" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="B20" t="s">
-        <x:v>62</x:v>
-      </x:c>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B20"/>
       <x:c r="C20"/>
       <x:c r="D20"/>
       <x:c r="E20"/>
@@ -1801,10 +1808,10 @@
     </x:row>
     <x:row r="21" ht="36.75" customHeight="1">
       <x:c r="A21" t="s">
-        <x:v>63</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B21" t="s">
-        <x:v>64</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C21"/>
       <x:c r="D21"/>
@@ -1815,12 +1822,12 @@
       <x:c r="I21"/>
       <x:c r="J21"/>
     </x:row>
-    <x:row r="22">
+    <x:row r="22" ht="36.75" customHeight="1">
       <x:c r="A22" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B22" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C22"/>
       <x:c r="D22"/>
@@ -1833,10 +1840,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="s">
-        <x:v>67</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B23" t="s">
-        <x:v>68</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C23"/>
       <x:c r="D23"/>
@@ -1849,10 +1856,10 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="s">
-        <x:v>69</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B24" t="s">
-        <x:v>70</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C24"/>
       <x:c r="D24"/>
@@ -1865,10 +1872,10 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B25" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C25"/>
       <x:c r="D25"/>
@@ -1880,8 +1887,12 @@
       <x:c r="J25"/>
     </x:row>
     <x:row r="26">
-      <x:c r="A26"/>
-      <x:c r="B26"/>
+      <x:c r="A26" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B26" t="s">
+        <x:v>72</x:v>
+      </x:c>
       <x:c r="C26"/>
       <x:c r="D26"/>
       <x:c r="E26"/>
@@ -2591,16 +2602,17 @@
         <x:v>Offensive Core 能否在不接入正式 Runtime 的前提下，同時支援一出局一壘與一出局二壘，並讓壘況具體改變決策、結果與跑者推進？</x:v>
       </x:c>
       <x:c r="D17" t="str">
-        <x:v>擴充精確 Base State API；建立 Base-State-aware Decision／Result／State Delta；保留一壘既有機率；新增二壘滾地、安打、觸擊與跑者推進模型；高中春季打擊僅由不相容改為 readiness-only compatible。</x:v>
+        <x:v>擴充精確 Base State API；建立 Base-State-aware Decision／Result／State Delta；保留一壘既有機率；新增二壘滾地、安打、觸擊與跑者推進模型；高中春季打擊僅由不相容改為 readiness-only。</x:v>
       </x:c>
       <x:c r="E17" t="str">
         <x:v>baseball-offense-prototype.js；baseball-gameplay-integration.js；Sandbox Base State selector；Offensive Base State tests；5.3 design document</x:v>
       </x:c>
       <x:c r="F17" t="str">
-        <x:v>支援 one-out-runner-on-first 與 one-out-runner-on-second；未知 Base State fail closed；runnersAfter 成為通用壘況真相；一壘回歸不變；二壘不產生一般雙殺或野選；正式 Player／Save／Story／Runtime mutation 維持不變。</x:v>
+        <x:v>支援 one-out-runner-on-first 與 one-out-runner-on-second；未知 Base State fail closed；runnersAfter 成為通用壘況真相；一壘回歸不變；二壘結果符合棒球規則。</x:v>
       </x:c>
       <x:c r="G17" t="str">
         <x:v>起始基線：028cffb
+結案基線：3b50316
 Gameplay Test Level B+
 Offensive Base-State Model Expansion</x:v>
       </x:c>
@@ -2608,33 +2620,51 @@
         <x:v>完成</x:v>
       </x:c>
     </x:row>
-    <x:row r="18">
+    <x:row r="18" ht="116" customHeight="1">
       <x:c r="A18" t="str">
+        <x:v>5.4</x:v>
+      </x:c>
+      <x:c r="B18" t="str">
+        <x:v>Gameplay Validation IV</x:v>
+      </x:c>
+      <x:c r="C18" t="str">
+        <x:v>二壘有人、一出局的高中春季打席能否首次安全接入正式 Runtime，並把 Core 結果 exactly once 寫入 Player Match State？</x:v>
+      </x:c>
+      <x:c r="D18" t="str">
+        <x:v>將 high_school_year_two_spring_game 改為 live offensive integration；四種具體打席策略由 Offensive Core 決策與執行；正式更新出局數、壘況、比分與球季表現；結果停留在 Outcome 等待玩家繼續。</x:v>
+      </x:c>
+      <x:c r="E18" t="str">
+        <x:v>baseball-gameplay-integration.js；script.js；story.js；tests/baseball-gameplay-integration-test.js；tests/baseball-gameplay-prototype-isolation-test.js；tests/high-school-three-year-spine-test.js；tests/baseball-offensive-production-integration-test.js；docs/gameplay-sprint-5.4-first-offensive-production-integration.md</x:v>
+      </x:c>
+      <x:c r="F18" t="str">
+        <x:v>one-out-runner-on-second 正式打席可完成；runnersAfter 是壘況真相；Core 不直接修改 Player；結果與策略旗標分離；pending Save fail closed；Outcome Continue 與少棒守備 pilot 均不回歸。</x:v>
+      </x:c>
+      <x:c r="G18" t="str">
+        <x:v>起始基線：3b50316
+Gameplay Test Level C
+First Production Offensive Mutation Integration</x:v>
+      </x:c>
+      <x:c r="H18" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" t="str">
         <x:v>4.13+</x:v>
       </x:c>
-      <x:c r="B18"/>
-      <x:c r="C18" t="str">
+      <x:c r="B19"/>
+      <x:c r="C19" t="str">
         <x:v>Post-Age-22 Architecture Expansion／Deferred pending Gameplay Validation</x:v>
       </x:c>
-      <x:c r="D18"/>
-      <x:c r="E18"/>
-      <x:c r="F18" t="str">
-        <x:v>不排 Eligibility 施工日期；後續 Gameplay Sprint 日期未規劃。</x:v>
-      </x:c>
-      <x:c r="G18"/>
-      <x:c r="H18" t="str">
-        <x:v>延後</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19"/>
-      <x:c r="B19"/>
-      <x:c r="C19"/>
       <x:c r="D19"/>
       <x:c r="E19"/>
-      <x:c r="F19"/>
+      <x:c r="F19" t="str">
+        <x:v>不排 Eligibility 施工日期；後續 Gameplay Sprint 日期未規劃。</x:v>
+      </x:c>
       <x:c r="G19"/>
-      <x:c r="H19"/>
+      <x:c r="H19" t="str">
+        <x:v>延後</x:v>
+      </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20"/>

</xml_diff>

<commit_message>
feat: establish high school training rhythm prototype
</commit_message>
<xml_diff>
--- a/棒球人生_三年設計排程_易讀版.xlsx
+++ b/棒球人生_三年設計排程_易讀版.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="R6ac572880fa04d93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R87b4ad8228004c2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="R46ca32390d8f4a52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="R3d4b07bbbaec4b1c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="R19bc198f2bb04ecd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="Ra95f9b092aa4476d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="三年總覽" sheetId="1" r:id="R9b2d886d55624e6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="第一季甘特圖" sheetId="2" r:id="R4fdc0dc33c794f1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint驗收表" sheetId="3" r:id="Rb676612938d54fcd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作節奏" sheetId="4" r:id="Re4011bc8d36a4703"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="範圍禁區" sheetId="5" r:id="Rd6319fd93dee4f69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="先看這張" sheetId="6" r:id="R7771cd6b212346ea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1765,18 +1765,19 @@
         <x:v>起始基線：3b50316
 階段：Gameplay Validation IV
 核心工作：high_school_year_two_spring_game live integration；one-out-runner-on-second；Offensive Core → Player Match State。
-測試級別：Gameplay Test Level C／First Production Offensive Mutation Integration</x:v>
+測試級別：Gameplay Test Level C／First Production Offensive Mutation Integration
+結案基線：9bb2eb7</x:v>
       </x:c>
       <x:c r="J18" t="str">
         <x:v>完成</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="36.75" customHeight="1">
+    <x:row r="19" ht="92" customHeight="1">
       <x:c r="A19" s="20" t="str">
-        <x:v>4.13+</x:v>
+        <x:v>5.5</x:v>
       </x:c>
       <x:c r="B19" s="10" t="str">
-        <x:v>Post-Age-22 Architecture Expansion</x:v>
+        <x:v>Gameplay Sprint 5.5：Training Rhythm Prototype</x:v>
       </x:c>
       <x:c r="C19"/>
       <x:c r="D19"/>
@@ -1785,34 +1786,41 @@
       <x:c r="G19"/>
       <x:c r="H19"/>
       <x:c r="I19" t="str">
-        <x:v>Deferred pending Gameplay Validation
-目前不排 Eligibility 施工日期；後續 Gameplay Sprint 日期未規劃。</x:v>
+        <x:v>起始基線：9bb2eb7
+階段：Gameplay Validation V
+核心工作：高二春季前兩個 Production Training Slot；五種固定訓練；readonly Training Resolver；exactly-once Player mutation；Outcome Hold／Continue；既有 Gameplay source facts 可被準備選擇改變。
+測試級別：Gameplay Test Level C／Production Training Rhythm Prototype</x:v>
       </x:c>
       <x:c r="J19" t="str">
-        <x:v>延後</x:v>
+        <x:v>完成</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="36.75" customHeight="1">
-      <x:c r="A20" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="B20"/>
+      <x:c r="A20" t="str">
+        <x:v>4.13+</x:v>
+      </x:c>
+      <x:c r="B20" t="str">
+        <x:v>Post-Age-22 Architecture Expansion</x:v>
+      </x:c>
       <x:c r="C20"/>
       <x:c r="D20"/>
       <x:c r="E20"/>
       <x:c r="F20"/>
       <x:c r="G20"/>
       <x:c r="H20"/>
-      <x:c r="I20"/>
-      <x:c r="J20"/>
+      <x:c r="I20" t="str">
+        <x:v>Deferred pending Gameplay Validation
+目前不排 Eligibility 施工日期；後續 Gameplay Sprint 日期未規劃。</x:v>
+      </x:c>
+      <x:c r="J20" t="str">
+        <x:v>延後</x:v>
+      </x:c>
     </x:row>
     <x:row r="21" ht="36.75" customHeight="1">
       <x:c r="A21" t="s">
-        <x:v>61</x:v>
-      </x:c>
-      <x:c r="B21" t="s">
-        <x:v>62</x:v>
-      </x:c>
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B21"/>
       <x:c r="C21"/>
       <x:c r="D21"/>
       <x:c r="E21"/>
@@ -1824,10 +1832,10 @@
     </x:row>
     <x:row r="22" ht="36.75" customHeight="1">
       <x:c r="A22" t="s">
-        <x:v>63</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B22" t="s">
-        <x:v>64</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C22"/>
       <x:c r="D22"/>
@@ -1840,10 +1848,10 @@
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="s">
-        <x:v>65</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B23" t="s">
-        <x:v>66</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="C23"/>
       <x:c r="D23"/>
@@ -1856,10 +1864,10 @@
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="s">
-        <x:v>67</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B24" t="s">
-        <x:v>68</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="C24"/>
       <x:c r="D24"/>
@@ -1872,10 +1880,10 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="s">
-        <x:v>69</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B25" t="s">
-        <x:v>70</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="C25"/>
       <x:c r="D25"/>
@@ -1888,10 +1896,10 @@
     </x:row>
     <x:row r="26">
       <x:c r="A26" t="s">
-        <x:v>71</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B26" t="s">
-        <x:v>72</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="C26"/>
       <x:c r="D26"/>
@@ -1903,8 +1911,12 @@
       <x:c r="J26"/>
     </x:row>
     <x:row r="27">
-      <x:c r="A27"/>
-      <x:c r="B27"/>
+      <x:c r="A27" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="B27" t="s">
+        <x:v>72</x:v>
+      </x:c>
       <x:c r="C27"/>
       <x:c r="D27"/>
       <x:c r="E27"/>
@@ -2642,39 +2654,58 @@
       <x:c r="G18" t="str">
         <x:v>起始基線：3b50316
 Gameplay Test Level C
-First Production Offensive Mutation Integration</x:v>
+First Production Offensive Mutation Integration
+結案基線：9bb2eb7</x:v>
       </x:c>
       <x:c r="H18" t="str">
         <x:v>完成</x:v>
       </x:c>
     </x:row>
-    <x:row r="19">
+    <x:row r="19" ht="116" customHeight="1">
       <x:c r="A19" t="str">
+        <x:v>5.5</x:v>
+      </x:c>
+      <x:c r="B19" t="str">
+        <x:v>Gameplay Validation V</x:v>
+      </x:c>
+      <x:c r="C19" t="str">
+        <x:v>正式高中流程能否在不建立完整日曆或養成模式下，讓玩家於比賽前主動選擇準備方向，並讓既有 Gameplay Adapter 讀到改變後的能力與身體事實？</x:v>
+      </x:c>
+      <x:c r="D19" t="str">
+        <x:v>在青棒第二年春季聯賽前插入兩個一次性自主訓練時段；建立 readonly BaseballTrainingResolver；五種固定訓練 deterministic 結算；script.js exactly once 寫入 Player；結果停留等待 Continue；高二八幕 Career Spine 不變。</x:v>
+      </x:c>
+      <x:c r="E19" t="str">
+        <x:v>baseball-training-resolver.js；index.html；story.js；script.js；tests/baseball-training-rhythm-test.js；tests/high-school-three-year-spine-test.js；docs/gameplay-sprint-5.5-training-rhythm-prototype.md</x:v>
+      </x:c>
+      <x:c r="F19" t="str">
+        <x:v>Training A／B 各出現一次且不增加正式 step；五種訓練效果與疲勞取捨正確；contact／defense／body source facts 可改變既有 Adapter；未知訓練 fail closed；重複操作不重複套用；完成後可手動存檔；Player／Save／Career／5.4 公式不變。</x:v>
+      </x:c>
+      <x:c r="G19" t="str">
+        <x:v>起始基線：9bb2eb7
+Gameplay Test Level C
+Production Training Rhythm Prototype</x:v>
+      </x:c>
+      <x:c r="H19" t="str">
+        <x:v>完成</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" t="str">
         <x:v>4.13+</x:v>
       </x:c>
-      <x:c r="B19"/>
-      <x:c r="C19" t="str">
+      <x:c r="B20"/>
+      <x:c r="C20" t="str">
         <x:v>Post-Age-22 Architecture Expansion／Deferred pending Gameplay Validation</x:v>
       </x:c>
-      <x:c r="D19"/>
-      <x:c r="E19"/>
-      <x:c r="F19" t="str">
-        <x:v>不排 Eligibility 施工日期；後續 Gameplay Sprint 日期未規劃。</x:v>
-      </x:c>
-      <x:c r="G19"/>
-      <x:c r="H19" t="str">
-        <x:v>延後</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20"/>
-      <x:c r="B20"/>
-      <x:c r="C20"/>
       <x:c r="D20"/>
       <x:c r="E20"/>
-      <x:c r="F20"/>
+      <x:c r="F20" t="str">
+        <x:v>不排 Eligibility 施工日期；後續 Gameplay Sprint 日期未規劃。</x:v>
+      </x:c>
       <x:c r="G20"/>
-      <x:c r="H20"/>
+      <x:c r="H20" t="str">
+        <x:v>延後</x:v>
+      </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21"/>

</xml_diff>